<commit_message>
Fix trailing comma in lean.devices JSON; regenerate Excel (118 rows)
Trailing comma left after moving 3 devices to qual broke JSON parsing
in the Excel generator. Fixed and Excel updated to reflect current content.

https://claude.ai/code/session_019KwCcZLvcVY13HRSnpAd9T
</commit_message>
<xml_diff>
--- a/Ansprechpartner_Review.xlsx
+++ b/Ansprechpartner_Review.xlsx
@@ -4090,50 +4090,50 @@
       <c r="J100" s="2" t="inlineStr"/>
     </row>
     <row r="101" ht="60" customHeight="1">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>LEAN · 3D-Druck · KANBAN</t>
-        </is>
-      </c>
-      <c r="B101" s="3" t="inlineStr">
-        <is>
-          <t>Haptic Device / 3D-Eingabestift</t>
-        </is>
-      </c>
-      <c r="C101" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D101" s="3" t="inlineStr">
-        <is>
-          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="E101" s="3" t="inlineStr">
-        <is>
-          <t>Einweisung erforderlich</t>
-        </is>
-      </c>
-      <c r="F101" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G101" s="3" t="inlineStr"/>
-      <c r="H101" s="3" t="inlineStr"/>
-      <c r="I101" s="3" t="inlineStr"/>
-      <c r="J101" s="3" t="inlineStr"/>
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Qualifizierung · Einweisung</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>CAD/CAM Sicherheitseinweisung</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D101" s="5" t="inlineStr">
+        <is>
+          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
+        </is>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G101" s="5" t="inlineStr"/>
+      <c r="H101" s="5" t="inlineStr"/>
+      <c r="I101" s="5" t="inlineStr"/>
+      <c r="J101" s="5" t="inlineStr"/>
     </row>
     <row r="102" ht="60" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>LEAN · 3D-Druck · KANBAN</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Einweisung KanbanSlides Excel</t>
+          <t>Intraoralscanner (IOS) Einweisung</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -4143,17 +4143,17 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
+          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr"/>
@@ -4164,12 +4164,12 @@
     <row r="103" ht="60" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>LEAN · 3D-Druck · KANBAN</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>KANBAN Materialverwaltung</t>
+          <t>Design-Prozess 4./5. Fachsemester</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -4179,17 +4179,17 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
+          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Zahnärztlicher Kollege</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Zuständigen zahnärztlichen Kollegen ansprechen</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr"/>
@@ -4198,40 +4198,40 @@
       <c r="J103" s="3" t="inlineStr"/>
     </row>
     <row r="104" ht="60" customHeight="1">
-      <c r="A104" s="2" t="inlineStr">
+      <c r="A104" s="4" t="inlineStr">
         <is>
           <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>CAD/CAM Sicherheitseinweisung</t>
-        </is>
-      </c>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
-        </is>
-      </c>
-      <c r="E104" s="2" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr"/>
-      <c r="I104" s="2" t="inlineStr"/>
-      <c r="J104" s="2" t="inlineStr"/>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>Schulungsvideos / Kompetenzmatrix</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>(1) Auf ILIAS nach Schulungsvideos &amp; Kompetenzmatrix suchen → (2) Vor Gerätenutzung relevante Videos ansehen</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F104" s="4" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr"/>
+      <c r="H104" s="4" t="inlineStr"/>
+      <c r="I104" s="4" t="inlineStr"/>
+      <c r="J104" s="4" t="inlineStr"/>
     </row>
     <row r="105" ht="60" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Intraoralscanner (IOS) Einweisung</t>
+          <t>Slicing / Nesting für Kurse</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -4251,17 +4251,17 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
+          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr"/>
@@ -4277,7 +4277,7 @@
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Design-Prozess 4./5. Fachsemester</t>
+          <t>Medientechnik</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -4287,17 +4287,17 @@
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
+          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen → (2) Ohne Einweisung das Medienpanel nicht selbstständig bedienen</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>Zahnärztlicher Kollege</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>Zuständigen zahnärztlichen Kollegen ansprechen</t>
+          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr"/>
@@ -4313,7 +4313,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Schulungsvideos / Kompetenzmatrix</t>
+          <t>Haptic Device / 3D-Eingabestift</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -4323,17 +4323,17 @@
       </c>
       <c r="D107" s="3" t="inlineStr">
         <is>
-          <t>(1) Auf ILIAS nach Schulungsvideos &amp; Kompetenzmatrix suchen → (2) Vor Gerätenutzung relevante Videos ansehen</t>
+          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Einweisung erforderlich</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr"/>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Slicing / Nesting für Kurse</t>
+          <t>Einweisung KanbanSlides Excel</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -4359,17 +4359,17 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
+          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr"/>
@@ -4385,7 +4385,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Medientechnik</t>
+          <t>KANBAN Materialverwaltung</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -4395,17 +4395,17 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen → (2) Ohne Einweisung das Medienpanel nicht selbstständig bedienen</t>
+          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Apply reviewed contact/steps data from Ansprechpartner_Review.xlsx
- Update 113 existing devices with corrected AP1 contacts, contact-detail
  lines and self-help steps from the reviewed Excel
- Add 8 new devices: PC/Workstation Funktionsstörung in CAD-Raum,
  CAM-Raum and Besprechung Lehrende (3 new), plus Patientenkamera /
  in Seminar 3, Labcam/Demokamera and Kein-Strom in Technicum (3 new)
- Rename 'Ausstattung – analoger Raum' → 'Ausstattung – Lautsprecher'
  in Seminar 2, and 'Handstück' → 'Handstück dreht links' in Technicum
- Regenerate Ansprechpartner_Review.xlsx (now 124 rows)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KwCcZLvcVY13HRSnpAd9T
</commit_message>
<xml_diff>
--- a/Ansprechpartner_Review.xlsx
+++ b/Ansprechpartner_Review.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -558,18 +558,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>(1) Medienpanel in SR1 &amp; SR3 ausschalten, dann in SR1 einschalten (ca. 90 Sekunden) → (2) Cave: Nach Benutzung immer ausschalten.</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Arzt Skill Labs; Techn. Koordinator oder IT-Service Tal ansprechen</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
@@ -605,7 +609,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Serviceportal ggf. Emailaddresse hier hinterlegen</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr"/>
@@ -636,12 +640,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in Techn. Koordinator CC</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
@@ -667,12 +671,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC auf Input 1 zurückschalten -</t>
+          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC, Switch auf Input 1 schalten.-</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -703,17 +707,17 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Die Kurbel liegt für gewöhnlich in einem der Medienkoffer in SR1 oder SR3. → (2) Erklärvideo auf Q:\</t>
+          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Die Kurbel liegt für gewöhnlich in einem der Medienkoffer in SR1 oder SR3. → (2) Erklärvideo auf Q:</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
@@ -811,7 +815,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>(1) Ist der Projektor am Medienpanel eingeschaltet? → (2) Ist Bild Aus/Ein aktiviert (rot oder grün)? → (3) Ist die Bildquelle korrekt ausgewählt?</t>
+          <t>(1) Ist der Projektor am Medienpanel eingeschaltet? → (2) Ist Bild Aus/Ein aktiviert (rot oder grün)? → (3) Ist die Bildquelle korrekt ausgewählt? (4) Windowstaste+P klickenauf Account clicken und Dublizieren/Erweitern auswählen</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -852,7 +856,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -883,7 +887,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Neustart versuchen. → (7) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -893,7 +897,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
@@ -924,12 +928,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -945,7 +949,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Ausstattung – analoger Raum</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -955,11 +959,19 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>(1) Seminar 2 ist analog ausgestattet: Metaplan-Wand und Flipchart. Keine fest installierte AV-Technik. → (2) In diesem Raum befindet sich ein zusätzlicher Lautsprecher, welcher sich vom Medienpanel SR3 steuern lässt.</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+        </is>
+      </c>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
@@ -973,7 +985,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Ausstattung – Lautsprecher</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -983,19 +995,15 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Seminar 2 ist analog ausgestattet: Metaplan-Wand und Flipchart. Keine fest installierte AV-Technik. → (2) In diesem Raum befindet sich ein zusätzlicher Lautsprecher, welcher sich vom Medienpanel SR3 steuern lässt.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
-        </is>
-      </c>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr"/>
@@ -1017,15 +1025,19 @@
           <t>branch</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>(1) Medienpanel in SR1 &amp; SR3 ausschalten, dann in SR1 einschalten (ca. 90 Sekunden) → (2) Cave: Nach Benutzung immer ausschalten.</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
@@ -1092,7 +1104,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1128,12 +1140,12 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
@@ -1169,7 +1181,7 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
@@ -1200,12 +1212,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
@@ -1234,7 +1246,11 @@
           <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Erklärvideo auf Q:\</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Werkstatt ZMK</t>
+        </is>
+      </c>
       <c r="F21" s="3" t="inlineStr"/>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
@@ -1331,7 +1347,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Neustart versuchen. → (7) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -1341,7 +1357,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr"/>
@@ -1350,76 +1366,76 @@
       <c r="J24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Seminar 3</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Patientenkamera /</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>(1) Gerät über das Medienpanel kurz aus- und wieder einschalten → (2) Kabel- und Signalverbindung dewr Kamera prüfen</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Mit Einweisung → direkt kontaktieren | Ohne Einweisung → zuerst Techn. Koordinator</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Technicum</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Hotty Wax Station</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>(1) Temperatur je nach Wachstyp einstellen – mind. 10 Min. vorheizen lassen. → (2) Nur zugelassene Dentalwachse verwenden. → (3) Instrumente im Gerät reinigen, bevor die Arbeit beginnt. → (4) Nach Gebrauch: Gerät ausschalten, keine Wachsreste im Becken lassen.</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr"/>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Technicum</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Intraoralscanner</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -1429,7 +1445,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Sirona SIM Intego Bench</t>
+          <t>Intraoralscanner</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1439,7 +1455,7 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>(1) Fußschalter prüfen – eingesteckt und im richtigen Modus? → (2) Handstück einsetzen bis es hörbar einrastet. → (3) Wasser / Luft kommt nicht? Absperrventil am Gerät öffnen. → (4) Licht defekt? Handstücklampe prüfen (fest einschrauben). → (5) Gerät reagiert gar nicht? Hauptschalter an der Rückseite prüfen.</t>
+          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1465,23 +1481,27 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Medienpanel / Raumsteuerung</t>
+          <t>Sirona SIM Intego Bench</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>(1) Fußschalter prüfen – eingesteckt und im richtigen Modus? → (2) Handstück einsetzen bis es hörbar einrastet. → (3) Wasser / Luft kommt nicht? Absperrventil am Gerät öffnen. → (4) Licht defekt? Handstücklampe prüfen (fest einschrauben). → (5) Gerät reagiert gar nicht? Hauptschalter an der Rückseite prüfen.</t>
+        </is>
+      </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr"/>
@@ -1497,39 +1517,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr"/>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>System einschalten lassen</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Aufsicht / Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Aufsicht / Assistenzarzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Im Raum „Besprechung Lehrende“ ansprechen</t>
-        </is>
-      </c>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
     </row>
@@ -1541,7 +1549,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Noflame Plus</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1551,17 +1559,17 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>(1) Instrument aus der Spulenöffnung nehmen → (2) Gerät aus- und wieder einschalten → (3) Lüftungsschlitze freiräumen → (4) Gerät ausschalten → (5) Einige Minuten abkühlen lassen → (6) Neu starten</t>
+          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr"/>
@@ -1577,17 +1585,17 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>QUATTROcare</t>
+          <t>Noflame Plus</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>(1) Ersatzkartuschen bei den Aufsichten. Kartuschen können selbst gewechselt werden.</t>
+          <t>(1) Instrument aus der Spulenöffnung nehmen → (2) Gerät aus- und wieder einschalten → (3) Lüftungsschlitze freiräumen → (4) Gerät ausschalten → (5) Einige Minuten abkühlen lassen → (6) Neu starten</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1597,7 +1605,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1613,7 +1621,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Demokamera</t>
+          <t>QUATTROcare</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1623,17 +1631,17 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC auf Input 1 zurückschalten -</t>
+          <t>(1) Ersatzkartuschen bei den Aufsichten. Kartuschen können selbst gewechselt werden.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Einweisung erforderlich</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
@@ -1649,7 +1657,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Bildschirme schwarz</t>
+          <t>Demokamera</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1659,17 +1667,17 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>(1) Am Medienpanel richtiges Signal ausgewählt? → (2) Signal neu zuweisen. → (3) Bildschirm am Panel aus- und wieder einschalten</t>
+          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC auf Input 1 zurückschalten -</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Einweisung erforderlich</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
@@ -1685,7 +1693,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Notschalter ausgelöst</t>
+          <t>Bildschirme schwarz</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1695,17 +1703,17 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>(1) Prüfen ob der Auslösegrund behoben ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
+          <t>(1) Am Medienpanel richtiges Signal ausgewählt? → (2) Signal neu zuweisen. → (3) Bildschirm am Panel aus- und wieder einschalten</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr"/>
@@ -1721,7 +1729,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>Notschalter ausgelöst</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1731,17 +1739,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
+          <t>(1) Prüfen ob der Auslösegrund behoben ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr"/>
@@ -1757,7 +1765,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -1767,17 +1775,17 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
@@ -1793,7 +1801,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Handstück</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -1803,17 +1811,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>(1) Fehler F5: Kniesteuerung komplett ausschalten (10s warten) → (2) Linkslauf: Gerät ist im Linksbetrieb! → (3) Am Netzschalter (11) ausschalten → (4) Rechtslauftaste T4 (Plustaste) gedrückt halten → (5) Dabei Netzschalter wieder einschalten → (6) LED T3 aus = Rechtslauf aktiv</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr"/>
@@ -1849,7 +1857,7 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr"/>
@@ -1908,12 +1916,12 @@
       <c r="D40" s="4" t="inlineStr"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen</t>
+          <t>Arzt im Raum „Besprechung Lehrende“ ansprechen</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
@@ -1939,7 +1947,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Neustart versuchen. → (7) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
@@ -1949,7 +1957,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr"/>
@@ -1958,50 +1966,50 @@
       <c r="J41" s="3" t="inlineStr"/>
     </row>
     <row r="42" ht="60" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Phantomicum</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Arbeitsplatzkamera</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>(1) Kamera einschalten, USB-Verbindung zum Rechner prüfen. → (2) Richtige Kameraquelle in der Software auswählen. → (3) Kein Bild? Software neu starten, Kabel neu einstecken.</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="2" t="inlineStr"/>
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Technicum</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Labcam / Demokamera</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC, Switch auf Input 1 schalten.-</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Phantomicum</t>
+          <t>Technicum</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Intraoralscanner</t>
+          <t>Kein Strom an allen Plätzen</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2011,7 +2019,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
+          <t>(1) Prüfen ob der Auslösegrund behoben ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2021,7 +2029,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr"/>
@@ -2032,12 +2040,12 @@
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Phantomicum</t>
+          <t>Technicum</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Pentamix 3</t>
+          <t>Handstück dreht links</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2047,7 +2055,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>(1) Bedienung im Kurs nach Einführung selbstständig.</t>
+          <t>(1) Fehler F5: Kniesteuerung komplett ausschalten (10s warten) → (2) Linkslauf: Gerät ist im Linksbetrieb! → (3) Am Netzschalter (11) ausschalten → (4) Rechtslauftaste T4 (Plustaste) gedrückt halten → (5) Dabei Netzschalter wieder einschalten → (6) LED T3 aus = Rechtslauf aktiv</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -2057,7 +2065,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr"/>
@@ -2066,36 +2074,40 @@
       <c r="J44" s="4" t="inlineStr"/>
     </row>
     <row r="45" ht="60" customHeight="1">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Phantomicum</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Medienpanel / Raumsteuerung</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr"/>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr"/>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Arbeitsplatzkamera</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>(1) Richtige Kameraquelle am Panel ausgewählt (2) NDI-PC gestartet? → (2) Notschalter an?</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -2105,17 +2117,17 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Behandlungseinheit / Turbine / Handstück</t>
+          <t>Intraoralscanner</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>(1) Ist die Behandlungseinheit eingeschaltet? → (2) Druckluft- und Wasser-Haupthahn geöffnet? → (3) Handstück/Turbine korrekt aufgesteckt und eingerastet? → (4) Einheit kurz aus- und wieder einschalten → (5) Lichtschalter an der Einheit betätigt? → (6) Helligkeit am Bedienfeld geprüft? → (7) Einheit aus- und wieder einschalten → (8) Haupthahn für Wasser und Druckluft geöffnet? → (9) Fußanlasser betätigt? → (10) Schläuche korrekt angeschlossen und nicht geknickt?</t>
+          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2125,7 +2137,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
@@ -2141,7 +2153,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>QUATTROcare</t>
+          <t>Pentamix 3</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2151,7 +2163,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>(1) Ersatzkartuschen bei den Aufsichten. Handstückpflege durch Studierende selbst.</t>
+          <t>(1) Bedienung im Kurs nach Einführung selbstständig.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2161,7 +2173,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Sekretariat / Koordination Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr"/>
@@ -2177,27 +2189,23 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Cavex Alginate Mixer</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>(1) Bedienung im Kurs nach Einführung durch Aufsichten selbstständig.</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
@@ -2213,27 +2221,27 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Behandlungseinheit / Turbine / Handstück</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Ist die Behandlungseinheit eingeschaltet? → (2) Druckluft- und Wasser-Haupthahn geöffnet? → (3) Handstück/Turbine korrekt aufgesteckt und eingerastet? → (4) Einheit kurz aus- und wieder einschalten → (5) Lichtschalter an der Einheit betätigt? → (6) Helligkeit am Bedienfeld geprüft? → (7) Einheit aus- und wieder einschalten → (8) Haupthahn für Wasser und Druckluft geöffnet? → (9) Fußanlasser betätigt? → (10) Schläuche korrekt angeschlossen und nicht geknickt?</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr"/>
@@ -2249,27 +2257,27 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>PC / Workstation – Funktionsstörung</t>
+          <t>QUATTROcare</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Neustart versuchen. → (7) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Ersatzkartuschen bei den Aufsichten. Handstückpflege durch Studierende selbst.</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
@@ -2278,50 +2286,50 @@
       <c r="J50" s="4" t="inlineStr"/>
     </row>
     <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Gipsen &amp; Polieren</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>Absaugbox BIOSTEAM Center</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>(1) Hauptschalter drücken – Gerät läuft, sobald Absaugung aktiv ist (hörbar). → (2) Schlauch auf Knickstellen oder Verstopfungen prüfen. → (3) Saugleistung schwach? Filter / Sieb prüfen und ggf. reinigen. → (4) Wasserbehälter entleeren wenn Füllstand-Anzeige leuchtet.</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Phantomicum</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Cavex Alginate Mixer</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>(1) Bedienung im Kurs nach Einführung durch Aufsichten selbstständig.</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr"/>
-      <c r="H51" s="5" t="inlineStr"/>
-      <c r="I51" s="5" t="inlineStr"/>
-      <c r="J51" s="5" t="inlineStr"/>
+      <c r="G51" s="3" t="inlineStr"/>
+      <c r="H51" s="3" t="inlineStr"/>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Gipsen &amp; Polieren</t>
+          <t>Phantomicum</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Steamy Mini (Abdampfer)</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -2331,17 +2339,17 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>(1) Wassertank befüllen (destilliertes Wasser – nur bei abgekühltem Gerät). → (2) Aufheizzeit abwarten – ca. 3–5 Min. bis Betriebsdruck erreicht ist. → (3) Düse verstopft? Nadel aus dem Zubehör vorsichtig durchstecken. → (4) Nach Gebrauch: Ausschalten, Restdampf ablassen.</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
@@ -2352,32 +2360,32 @@
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Gipsen &amp; Polieren</t>
+          <t>Phantomicum</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Trockentrimmer</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>(1) Hauptschalter prüfen – Absaugung muss laufen (hörbar), erst dann trimmen. → (2) Modell flach und gerade aufsetzen, gleichmäßigen Druck ausüben – nicht verkanten. → (3) Sollte das Schleifband verrutscht sein, bitte nicht selbst reparieren.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr"/>
@@ -2386,40 +2394,40 @@
       <c r="J53" s="3" t="inlineStr"/>
     </row>
     <row r="54" ht="60" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>Erkoform 3d motion</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>(1) Folientyp und -stärke laut Kursanleitung wählen (Aufkleber am Gerät beachten). → (2) Folie sorgfältig einspannen – Rahmen gleichmäßig und fest schließen. → (3) Temperatur und Druck je nach Material einstellen. → (4) Folie reißt? Temperatur oder Foliendicke prüfen, ggf. neu einspannen. → (5) Nach Abkühlung Modell entnehmen, Folie vorsichtig abtrennen.</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Absaugbox BIOSTEAM Center</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>(1) Hauptschalter drücken – Gerät läuft, sobald Absaugung aktiv ist (hörbar). → (2) Schlauch auf Knickstellen oder Verstopfungen prüfen. → (3) Saugleistung schwach? Filter / Sieb prüfen und ggf. reinigen. → (4) Wasserbehälter entleeren wenn Füllstand-Anzeige leuchtet.</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr"/>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -2429,7 +2437,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Giroform</t>
+          <t>Steamy Mini (Abdampfer)</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -2439,7 +2447,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>(1) Nur nach erfolgter Einweisung verwenden. → (2) Stiftposition nach Kursanleitung wählen – Stifte korrekt einsetzen und sichern. → (3) Modell in Artikulator einsetzen: Index-Stifte korrekt ausrichten und einrasten lassen.</t>
+          <t>(1) Wassertank befüllen (destilliertes Wasser – nur bei abgekühltem Gerät). → (2) Aufheizzeit abwarten – ca. 3–5 Min. bis Betriebsdruck erreicht ist. → (3) Düse verstopft? Nadel aus dem Zubehör vorsichtig durchstecken. → (4) Nach Gebrauch: Ausschalten, Restdampf ablassen.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -2465,7 +2473,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Smartbox X2</t>
+          <t>Trockentrimmer</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -2475,7 +2483,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>(1) Wasser einfüllen, Gerät einschalten – Vorheizzeit ca. 5 Min. abwarten. → (2) Küvette einlegen, Deckel fest verschließen – O-Ring auf Sauberkeit prüfen. → (3) Druck und Zeit gemäß Kursanleitung einstellen. → (4) Nach Ende: Druck über Ablassventil langsam ablassen, erst dann öffnen.</t>
+          <t>(1) Hauptschalter prüfen – Absaugung muss laufen (hörbar), erst dann trimmen. → (2) Modell flach und gerade aufsetzen, gleichmäßigen Druck ausüben – nicht verkanten. → (3) Sollte das Schleifband verrutscht sein, bitte nicht selbst reparieren.</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2501,7 +2509,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Smartmix</t>
+          <t>Erkoform 3d motion</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2511,7 +2519,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>(1) Schüssel und Paddel korrekt einsetzen und verriegeln. → (2) Wasser-Pulver-Verhältnis nach Anleitung abmessen (Messbecher verwenden). → (3) Mischzeit je nach Material einstellen (Gips ca. 30–45 s, Alginat ca. 45–60 s). → (4) Nach Gebrauch Schüssel und Paddel sofort reinigen.</t>
+          <t>(1) Folientyp und -stärke laut Kursanleitung wählen (Aufkleber am Gerät beachten). → (2) Folie sorgfältig einspannen – Rahmen gleichmäßig und fest schließen. → (3) Temperatur und Druck je nach Material einstellen. → (4) Folie reißt? Temperatur oder Foliendicke prüfen, ggf. neu einspannen. → (5) Nach Abkühlung Modell entnehmen, Folie vorsichtig abtrennen.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -2537,7 +2545,7 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Polierbox</t>
+          <t>Giroform</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -2547,7 +2555,7 @@
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>(1) Absaugung einschalten – Schalter am Gerät oder Fußpedal prüfen. → (2) Drehzahl am Handstück je nach Werkstück wählen. → (3) Saugleistung schwach? Filterbeutel / Sieb prüfen und ggf. reinigen. → (4) Handstück und Schleifkörper nach Nutzung reinigen.</t>
+          <t>(1) Nur nach erfolgter Einweisung verwenden. → (2) Stiftposition nach Kursanleitung wählen – Stifte korrekt einsetzen und sichern. → (3) Modell in Artikulator einsetzen: Index-Stifte korrekt ausrichten und einrasten lassen.</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -2573,39 +2581,31 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>Smartbox X2</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
+          <t>(1) Wasser einfüllen, Gerät einschalten – Vorheizzeit ca. 5 Min. abwarten. → (2) Küvette einlegen, Deckel fest verschließen – O-Ring auf Sauberkeit prüfen. → (3) Druck und Zeit gemäß Kursanleitung einstellen. → (4) Nach Ende: Druck über Ablassventil langsam ablassen, erst dann öffnen.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>System einschalten lassen</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>Aufsicht / Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t>Aufsicht / Assistenzarzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr">
-        <is>
-          <t>Im Raum „Besprechung Lehrende“ ansprechen</t>
-        </is>
-      </c>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr"/>
       <c r="I59" s="3" t="inlineStr"/>
       <c r="J59" s="3" t="inlineStr"/>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Abdampfgerät D-S100A</t>
+          <t>Smartmix</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>(1) Wasserhahn aufgedreht? → (2) Wasserstand im zweiten Abdampfer prüfen – ggf. nachfüllen</t>
+          <t>(1) Schüssel und Paddel korrekt einsetzen und verriegeln. → (2) Wasser-Pulver-Verhältnis nach Anleitung abmessen (Messbecher verwenden). → (3) Mischzeit je nach Material einstellen (Gips ca. 30–45 s, Alginat ca. 45–60 s). → (4) Nach Gebrauch Schüssel und Paddel sofort reinigen.</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Gipstrimmer HSS-88</t>
+          <t>Polierbox</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>(1) Ist der Wasserhahn aufgedreht? Das ist der häufigste Grund.</t>
+          <t>(1) Absaugung einschalten – Schalter am Gerät oder Fußpedal prüfen. → (2) Drehzahl am Handstück je nach Werkstück wählen. → (3) Saugleistung schwach? Filterbeutel / Sieb prüfen und ggf. reinigen. → (4) Handstück und Schleifkörper nach Nutzung reinigen.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -2689,17 +2689,17 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Rüttler</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>(1) Ein/Aus-Schalter und Intensitätsregler prüfen.</t>
+          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr"/>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Elmasonic S (Ultraschall)</t>
+          <t>Abdampfgerät D-S100A</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>(1) Wasser bis zur Markierung nachfüllen, dann neu starten.</t>
+          <t>(1) Wasserhahn aufgedreht? → (2) Wasserstand im zweiten Abdampfer prüfen – ggf. nachfüllen</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Erkoform 3d+</t>
+          <t>Gipstrimmer HSS-88</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>(1) Nur nach erfolgter Einweisung bedienen → (2) Folie und Einstellungen nach Kursanleitung wählen → (3) Bei Unsicherheit Einweisung anfordern</t>
+          <t>(1) Ist der Wasserhahn aufgedreht? Das ist der häufigste Grund.</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>Rüttler</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
+          <t>(1) Ein/Aus-Schalter und Intensitätsregler prüfen.</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
@@ -2833,27 +2833,27 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Gipsabscheider</t>
+          <t>Elmasonic S (Ultraschall)</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät nicht selbst öffnen oder entleeren. → (2) Füllstand / Störmeldung notieren. → (3) Werkstatt ZMK oder Technischen Koordinator informieren.</t>
+          <t>(1) Wasser bis zur Markierung nachfüllen, dann neu starten.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
@@ -2862,114 +2862,106 @@
       <c r="J66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="60" customHeight="1">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Gießen &amp; Strahlen</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>Augenspülstation</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Bei Spritzern ins Auge sofort ausgiebig mit der Augenspülstation spülen (mind. 30 s) und Lehrpersonal informieren. → (2) Standort: im Raum Gießen &amp; Strahlen. Betroffenes Auge sofort und ausgiebig spülen, Augenlid offen halten. Anschließend Lehrpersonal informieren und – außer bei Bagatelle – Unfallmeldung ausfüllen. Station stets frei zugänglich halten; Verfallsdatum der Spülflaschen beachten. → (3) Keine Gewähr der Angaben</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F67" s="5" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="inlineStr"/>
-      <c r="H67" s="5" t="inlineStr"/>
-      <c r="I67" s="5" t="inlineStr"/>
-      <c r="J67" s="5" t="inlineStr"/>
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Gipsen &amp; Polieren</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Erkoform 3d+</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>(1) Nur nach erfolgter Einweisung bedienen → (2) Folie und Einstellungen nach Kursanleitung wählen → (3) Bei Unsicherheit Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr"/>
+      <c r="I67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Gießen &amp; Strahlen</t>
+          <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>System einschalten lassen</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Aufsicht / Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>Aufsicht / Assistenzarzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="H68" s="4" t="inlineStr">
-        <is>
-          <t>Im Raum „Besprechung Lehrende“ ansprechen</t>
-        </is>
-      </c>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr"/>
+      <c r="H68" s="4" t="inlineStr"/>
       <c r="I68" s="4" t="inlineStr"/>
       <c r="J68" s="4" t="inlineStr"/>
     </row>
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Gießen &amp; Strahlen</t>
+          <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>eyevolution max</t>
+          <t>Gipsabscheider</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>(1) Ein/Aus-Schalter prüfen, Gerät neu starten. Am Strom angeschlossen? → (2) Programm nach Kursanleitung anpassen.</t>
+          <t>(1) Gerät nicht selbst öffnen oder entleeren. → (2) Füllstand / Störmeldung notieren.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr.</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr"/>
@@ -2978,40 +2970,40 @@
       <c r="J69" s="3" t="inlineStr"/>
     </row>
     <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>Sandstrahl BA9001</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>(1) Druckluftanschluss prüfen – ist der Hahn geöffnet? → (2) Düse vorsichtig nach Kursanleitung reinigen. → (3) Sand nach Kursanleitung nachfüllen. → (4) Kabinenfenster von innen reinigen.</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="inlineStr"/>
-      <c r="H70" s="4" t="inlineStr"/>
-      <c r="I70" s="4" t="inlineStr"/>
-      <c r="J70" s="4" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Augenspülstation</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Bei Spritzern ins Auge sofort ausgiebig mit der Augenspülstation spülen (mind. 30 s) und Lehrpersonal informieren. → (2) Standort: im Raum Gießen &amp; Strahlen. Betroffenes Auge sofort und ausgiebig spülen, Augenlid offen halten. Anschließend Lehrpersonal informieren und – außer bei Bagatelle – Unfallmeldung ausfüllen. Station stets frei zugänglich halten; Verfallsdatum der Spülflaschen beachten. → (3) Keine Gewähr der Angaben</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="60" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -3021,17 +3013,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Drucktopf</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Den Drucktopf niemals ohne vollständige Einweisung öffnen – immer erst Druck vollständig ablassen!</t>
+          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -3041,7 +3033,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr"/>
@@ -3057,7 +3049,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>eyevolution max</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3067,7 +3059,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
+          <t>(1) Ein/Aus-Schalter prüfen, Gerät neu starten. Am Strom angeschlossen? → (2) Programm nach Kursanleitung anpassen.</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3086,70 +3078,70 @@
       <c r="J72" s="4" t="inlineStr"/>
     </row>
     <row r="73" ht="60" customHeight="1">
-      <c r="A73" s="5" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>IO Scanner / Ceramill Map DRS</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>(1) Siehe laminierte Anleitung. → (2) Scanner-Status prüfen (eingeschaltet, angemeldet)</t>
-        </is>
-      </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="inlineStr"/>
-      <c r="H73" s="5" t="inlineStr"/>
-      <c r="I73" s="5" t="inlineStr"/>
-      <c r="J73" s="5" t="inlineStr"/>
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Gießen &amp; Strahlen</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Sandstrahl BA9001</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>(1) Druckluftanschluss prüfen – ist der Hahn geöffnet? → (2) Düse vorsichtig nach Kursanleitung reinigen. → (3) Sand nach Kursanleitung nachfüllen. → (4) Kabinenfenster von innen reinigen.</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="60" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination</t>
+          <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>KANBAN-Bestellung aufgeben</t>
+          <t>Drucktopf</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>(1) Karte an der KANBAN-Station im Sekretariat/ Koordination einlegen. → (2) Bearbeitung erfolgt automatisch.</t>
+          <t>(1) ⚠ Den Drucktopf niemals ohne Einweisung bedienen – immer erst Druck vollständig ablassen!</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr"/>
@@ -3160,12 +3152,12 @@
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination</t>
+          <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Laptops für Aufsichten</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3175,17 +3167,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>(1) Laptop im Sekretariat Skill Labs abholen. → (2) Einschalten und auf Funktionsfähigkeit prüfen. → (3) Nach dem Einsatz laden und zurückgeben.</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr"/>
@@ -3196,22 +3188,22 @@
     <row r="76" ht="60" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Papier &amp; Druck</t>
+          <t>Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Drucker</t>
+          <t>IO Scanner / Ceramill Map DRS</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>(1) Papierstau kann selbst behoben werden – Anleitung am Gerät. → (2) Tonerbestellung läuft automatisch. Kein Handlungsbedarf. → (3) Drucker aus- und wieder einschalten → (4) Am PC: Drucker ZM11 hinzufügen über 90_Wartung im Windows Menü → (5) Fehlermeldung am Display notieren → (6) Hält der Defekt an → Druckerwartung melden → (7) Windows Startmenü öffnen → Ordner 90_Wartung. → (8) Drucker ZM11 (oder gewünschten Drucker) aus der Liste auswählen und installieren. → (9) Nach Installation: Drucker ggf. als Standard festlegen.</t>
+          <t>(1) Siehe laminierte Anleitung. → (2) Scanner-Status prüfen (eingeschaltet, angemeldet)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3221,7 +3213,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Druckerwartung · Firma Morgenstern</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
@@ -3232,12 +3224,12 @@
     <row r="77" ht="60" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Papier &amp; Druck</t>
+          <t>Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Demoboxen</t>
+          <t>KANBAN-Bestellung aufgeben</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3247,89 +3239,85 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>(1) Nur für den Prothetik-Kurs vorgesehen → (2) Entnahme/Rückgabe mit der Koordination abstimmen</t>
+          <t>(1) Karte an der KANBAN-Station im Sekretariat/ Koordination einlegen. → (2) Bearbeitung erfolgt automatisch.</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="F77" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen</t>
-        </is>
-      </c>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
       <c r="G77" s="3" t="inlineStr"/>
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr"/>
       <c r="J77" s="3" t="inlineStr"/>
     </row>
     <row r="78" ht="60" customHeight="1">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>Besprechung Lehrende</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Küche &amp; Kaffee</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>(1) Mikrowelle, Kühlschrank und Kaffeevollautomat für Lehrende. Spül- und Reinigungsdienst für Tisch/Theke beachten – Organisation durch das Prothetik-Team.</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt im Raum „Besprechung Lehrende“ ansprechen | Falls nötig in CC / 2. Stelle: Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr"/>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="2" t="inlineStr"/>
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Laptops für Aufsichten</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>(1) Laptop im Sekretariat Skill Labs abholen. → (2) Einschalten und auf Funktionsfähigkeit prüfen. → (3) Nach dem Einsatz zurückgeben und zum laden einstecken.</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr"/>
+      <c r="H78" s="4" t="inlineStr"/>
+      <c r="I78" s="4" t="inlineStr"/>
+      <c r="J78" s="4" t="inlineStr"/>
     </row>
     <row r="79" ht="60" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>CAD-Raum</t>
+          <t>Papier &amp; Druck</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>3D-Scanner Pritimirror</t>
+          <t>Drucker</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>(1) Software starten, Scanner einschalten – grüne Status-LED abwarten. → (2) Kalibrierung prüfen – Software meldet bei veralteter Kalibrierung. → (3) Scanfläche sauber halten – Staubpartikel verfälschen das Ergebnis. → (4) Modell fest positionieren – Bewegung während des Scans vermeiden.</t>
+          <t>(1) Papierstau kann selbst behoben werden – Anleitung am Gerät. → (2) Tonerbestellung läuft automatisch. Kein Handlungsbedarf. (5) Fehlermeldung am Display notieren → (3) Hält der Defekt an → Druckerwartung melden → (4) Windows Startmenü öffnen → Ordner 90_Wartung. → (5) Drucker ZM11 (oder gewünschten Drucker) aus der Liste auswählen und installieren. → (6) Nach Installation: Drucker ggf. als Standard festlegen.</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Druckerwartung · Firma Morgenstern</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr"/>
@@ -3340,12 +3328,12 @@
     <row r="80" ht="60" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>CAD-Raum</t>
+          <t>Papier &amp; Druck</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Creality Scan Ferret</t>
+          <t>Demoboxen</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -3355,89 +3343,85 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>(1) USB-Kabel fest einstecken – Treiber werden beim ersten Start installiert. → (2) Scanner parallel zur Oberfläche halten, gleichmäßig und ruhig bewegen. → (3) Tracking verloren? Scan pausieren, Gerät näher an Oberfläche führen, neu starten.</t>
+          <t>(1) Nur für den Prothetik-Kurs vorgesehen → (2) Entnahme/Rückgabe mit der Koordination abstimmen</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr"/>
       <c r="G80" s="4" t="inlineStr"/>
       <c r="H80" s="4" t="inlineStr"/>
       <c r="I80" s="4" t="inlineStr"/>
       <c r="J80" s="4" t="inlineStr"/>
     </row>
     <row r="81" ht="60" customHeight="1">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>CAD-Raum</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>Laborscanner Ceramill Map 300</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>(1) Software öffnen (Ceramill Map), Scanner einschalten – Verbindung abwarten. → (2) Modell auf den Scantisch legen – Referenzpunkte nicht verdecken. → (3) Kalibrierung: bei Aufforderung Kalibriermodell verwenden.</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="inlineStr">
-        <is>
-          <t>Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
-      <c r="G81" s="3" t="inlineStr"/>
-      <c r="H81" s="3" t="inlineStr"/>
-      <c r="I81" s="3" t="inlineStr"/>
-      <c r="J81" s="3" t="inlineStr"/>
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Besprechung Lehrende</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Küche &amp; Kaffee</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>(1) Mikrowelle, Kühlschrank und Kaffeevollautomat für Lehrende. Spül- und Reinigungsdienst für Tisch/Theke beachten – Organisation durch das Prothetik-Team.</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Die Steuerung für die Zentralabsauguing/ Trockenabsaugung befindet sich in diesem Raum</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
+      <c r="I81" s="5" t="inlineStr"/>
+      <c r="J81" s="5" t="inlineStr"/>
     </row>
     <row r="82" ht="60" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>CAD-Raum</t>
+          <t>Besprechung Lehrende</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Haptic Pen (Geomagic Touch X)</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät per USB anschließen, dann Software starten (nicht umgekehrt). → (2) Arm in Ruheposition (Dock) halten beim Starten der Software. → (3) Bewegungsbereich frei halten – Kabel nicht knicken oder verknoten. → (4) Kalibrierung: Anweisungen in der Software folgen wenn aufgefordert.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -3446,36 +3430,40 @@
       <c r="J82" s="4" t="inlineStr"/>
     </row>
     <row r="83" ht="60" customHeight="1">
-      <c r="A83" s="3" t="inlineStr">
+      <c r="A83" s="5" t="inlineStr">
         <is>
           <t>CAD-Raum</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>Medienpanel / Raumsteuerung</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr"/>
-      <c r="E83" s="3" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F83" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen</t>
-        </is>
-      </c>
-      <c r="G83" s="3" t="inlineStr"/>
-      <c r="H83" s="3" t="inlineStr"/>
-      <c r="I83" s="3" t="inlineStr"/>
-      <c r="J83" s="3" t="inlineStr"/>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>3D-Scanner Pritimirror</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>(1) Software starten, Scanner einschalten – grüne Status-LED abwarten. → (2) Kalibrierung prüfen – Software meldet bei veralteter Kalibrierung. → (3) Scanfläche sauber halten – Staubpartikel verfälschen das Ergebnis. → (4) Modell fest positionieren – Bewegung während des Scans vermeiden.</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="5" t="inlineStr"/>
+      <c r="I83" s="5" t="inlineStr"/>
+      <c r="J83" s="5" t="inlineStr"/>
     </row>
     <row r="84" ht="60" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -3485,7 +3473,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Software startet nicht</t>
+          <t>Creality Scan Ferret</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -3495,17 +3483,17 @@
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) Software neu starten → (3) Lizenzserver erreichbar? → (4) Netzwerkverbindung prüfen (ist eine Eingabe der Proxydaten notwendig?)</t>
+          <t>(1) USB-Kabel fest einstecken – Treiber werden beim ersten Start installiert. → (2) Scanner parallel zur Oberfläche halten, gleichmäßig und ruhig bewegen. → (3) Tracking verloren? Scan pausieren, Gerät näher an Oberfläche führen, neu starten.</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -3521,7 +3509,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Lizenz nicht verfügbar</t>
+          <t>Laborscanner Ceramill Map 300</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -3531,17 +3519,17 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) Prüfen ob die Netzwerk-/Serververbindung steht → (3) Software schließen und erneut öffnen</t>
+          <t>(1) Software öffnen (Ceramill Map), Scanner einschalten – Verbindung abwarten. → (2) Modell auf den Scantisch legen – Referenzpunkte nicht verdecken. → (3) Kalibrierung: bei Aufforderung Kalibriermodell verwenden.</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr"/>
@@ -3557,7 +3545,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>3D-Maus (3Dconnexion)</t>
+          <t>Haptic Pen (Geomagic Touch X)</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -3567,17 +3555,17 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>(1) USB-Stecker neu einstecken → (2) Anderen USB-Port testen → (3) Prüfen ob die 3Dconnexion-Software/Treiber läuft</t>
+          <t>(1) Gerät per USB anschließen, dann Software starten (nicht umgekehrt). → (2) Arm in Ruheposition (Dock) halten beim Starten der Software. → (3) Bewegungsbereich frei halten – Kabel nicht knicken oder verknoten. → (4) Kalibrierung: Anweisungen in der Software folgen wenn aufgefordert.</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr"/>
@@ -3593,27 +3581,23 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Prusa Mini (3×)</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr">
-        <is>
-          <t>(1) Druckbett sauber und nivelliert? → (2) Filament vorhanden und korrekt eingezogen? → (3) Druckauftrag erneut senden</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr"/>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>3D-Druck Mailbox</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr"/>
@@ -3629,7 +3613,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>IT / Netzwerkproblem</t>
+          <t>Software startet nicht</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -3639,7 +3623,7 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) Netzwerkkabel / Verbindung prüfen → (3) Über Windows-Menü auf 90_Wartung und dann Gruppenrichtlinie abrufen.</t>
+          <t>(1) PC neu starten → (2) Software neu starten → (3) Lizenzserver erreichbar? → (4) Netzwerkverbindung prüfen (ist eine Eingabe der Proxydaten notwendig?)</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -3647,11 +3631,7 @@
           <t>IT-Service Tal</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
+      <c r="F88" s="4" t="inlineStr"/>
       <c r="G88" s="4" t="inlineStr"/>
       <c r="H88" s="4" t="inlineStr"/>
       <c r="I88" s="4" t="inlineStr"/>
@@ -3665,7 +3645,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Lizenz nicht verfügbar</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -3675,89 +3655,85 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) PC neu starten → (2) Prüfen ob die Netzwerk-/Serververbindung steht → (3) Software schließen und erneut öffnen</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F89" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
-        </is>
-      </c>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr"/>
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="3" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr"/>
       <c r="J89" s="3" t="inlineStr"/>
     </row>
     <row r="90" ht="60" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>CAM-Raum</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Ceramill Matik (Fräsmaschine)</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Nur eingewiesene Personen dürfen die Ceramill Matik bedienen.</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr"/>
-      <c r="J90" s="2" t="inlineStr"/>
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>CAD-Raum</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>3D-Maus (3Dconnexion)</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>(1) USB-Stecker neu einstecken → (2) Anderen USB-Port testen → (3) Prüfen ob die 3Dconnexion-Software/Treiber läuft</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr"/>
+      <c r="H90" s="4" t="inlineStr"/>
+      <c r="I90" s="4" t="inlineStr"/>
+      <c r="J90" s="4" t="inlineStr"/>
     </row>
     <row r="91" ht="60" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>CAM-Raum</t>
+          <t>CAD-Raum</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Ceramill Therm3 (Sinterofen)</t>
+          <t>Prusa Mini (3×)</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Nur eingewiesene Assistenzärzte dürfen den Sinterofen bedienen.</t>
+          <t>(1) Druckbett sauber und nivelliert? → (2) Filament vorhanden und korrekt eingezogen? → (3) Druckauftrag erneut senden</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>3D-Druck Mailbox</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr"/>
@@ -3768,32 +3744,32 @@
     <row r="92" ht="60" customHeight="1">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>CAM-Raum</t>
+          <t>CAD-Raum</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>xTool S1 Laser</t>
+          <t>IT / Netzwerkproblem</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>(1) ⚠ Schutzbrille Pflicht! Laser darf ausschließlich vom Techn. Koordinator bedient werden.</t>
+          <t>(1) PC neu starten → (2) Netzwerkkabel / Verbindung prüfen → (3) Über Windows-Menü auf 90_Wartung und dann Gruppenrichtlinie abrufen.</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr"/>
@@ -3804,12 +3780,12 @@
     <row r="93" ht="60" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>CAM-Raum</t>
+          <t>CAD-Raum</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Formlabs / Form Wash / Form Cure</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -3819,17 +3795,17 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>(1) Resin vorhanden, Tank sauber? → (2) Wash-/Cure-Zeiten nach Anleitung einstellen → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr"/>
@@ -3840,32 +3816,32 @@
     <row r="94" ht="60" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>CAM-Raum</t>
+          <t>CAD-Raum</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Bambu Lab / Prusa Mini</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>(1) Druckbett sauber &amp; nivelliert, Filament eingezogen? → (2) Druckauftrag erneut senden → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr"/>
@@ -3874,40 +3850,40 @@
       <c r="J94" s="4" t="inlineStr"/>
     </row>
     <row r="95" ht="60" customHeight="1">
-      <c r="A95" s="3" t="inlineStr">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>CAM-Raum</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
-        <is>
-          <t>KANBAN-Bestellung aufgeben</t>
-        </is>
-      </c>
-      <c r="C95" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>(1) Karte ausfüllen und an KANBAN Station im Sekretariat/Koordination Skill Labs einlegen</t>
-        </is>
-      </c>
-      <c r="E95" s="3" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Ceramill Matik (Fräsmaschine)</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Nur eingewiesene Personen dürfen die Ceramill Matik bedienen.</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
         <is>
           <t>Einweisung anfordern</t>
         </is>
       </c>
-      <c r="F95" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G95" s="3" t="inlineStr"/>
-      <c r="H95" s="3" t="inlineStr"/>
-      <c r="I95" s="3" t="inlineStr"/>
-      <c r="J95" s="3" t="inlineStr"/>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr"/>
+      <c r="H95" s="5" t="inlineStr"/>
+      <c r="I95" s="5" t="inlineStr"/>
+      <c r="J95" s="5" t="inlineStr"/>
     </row>
     <row r="96" ht="60" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
@@ -3917,27 +3893,27 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Gefahrstoffentsorgung (IPA)</t>
+          <t>Ceramill Therm3 (Sinterofen)</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>(1) Anmeldeformular Sonderabfälle ausfüllen (Anzahl / Art) → (2) Formular freitags an die Sonderabfall-Mailbox senden (Abholung dienstags) → (3) Etiketten bedrucken (IPA = halogenfreie Lösungsmittel) → (4) Kanister bekleben: UN-Nr. horizontal, Gefahrstoffkleber Spitze nach oben → (5) Kanister in Gefahrstoffcontainer OS8/LFB (Pfortenschlüssel im Sekretariat) → (6) Leere Kanister: ausdampfen, Symbol durchstreichen, ohne Deckel in gelben Sack</t>
+          <t>(1) ⚠ Nur eingewiesene Personen dürfen den Sinterofen bedienen.</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -3953,27 +3929,27 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>IT / Software</t>
+          <t>xTool S1 Laser</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) An-/Abmeldung und Netzwerkverbindung prüfen → (3) Hält das Problem an → IT-Service Tal</t>
+          <t>(1) ⚠ Schutzbrille Pflicht!  Nur eingewiesene Personen dürfen den Sinterofen bedienen..</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr"/>
@@ -3989,27 +3965,27 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Unfall / Notfall</t>
+          <t>Formlabs / Form Wash / Form Cure</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>(1) ⚠ Bei Verletzungen: Ärzte im Haus rufen, bei Bedarf Notarzt. SOP Unfallanzeige UKT beachten. Vorgesetzten informieren. Auge sofort an der Augendusche spülen, dabei aufhalten. Danach Arzt aufsuchen. Feuerlöscher: 1× Schaum. CO₂ bei Elektronik- und Flüssigkeitsbränden. Fluchtwege freihalten.</t>
+          <t>(1) Resin vorhanden, Tank artefaktfrei? → (2) Wash-/Cure-Zeiten nach Anleitung einstellen → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>Sofortmaßnahme</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Ärzte im Haus rufen, bei Bedarf Notarzt | SOP Unfallanzeige UKT beachten | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -4025,7 +4001,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Bambu Lab / Prusa Mini</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4035,17 +4011,17 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Druckbett sauber, Filament eingezogen? → (2) Druckauftrag auf SD Karte → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr"/>
@@ -4054,86 +4030,86 @@
       <c r="J99" s="3" t="inlineStr"/>
     </row>
     <row r="100" ht="60" customHeight="1">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>LEAN · 3D-Druck · KANBAN</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>3D-Druck-Anfrage stellen</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>(1) STL-Datei vorbereiten (geschlossenes Volumen, korrekte Größe) → (2) Kurze Beschreibung + gewünschtes Material angeben → (3) An die 3D-Druck-Mailbox senden</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>3D-Druck Mailbox</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr"/>
-      <c r="I100" s="2" t="inlineStr"/>
-      <c r="J100" s="2" t="inlineStr"/>
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>CAM-Raum</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>KANBAN-Bestellung aufgeben</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>(1) Karte ausfüllen und an KANBAN Station im Sekretariat/Koordination Skill Labs einlegen</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr"/>
+      <c r="H100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="inlineStr"/>
+      <c r="J100" s="4" t="inlineStr"/>
     </row>
     <row r="101" ht="60" customHeight="1">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t>Qualifizierung · Einweisung</t>
-        </is>
-      </c>
-      <c r="B101" s="5" t="inlineStr">
-        <is>
-          <t>CAD/CAM Sicherheitseinweisung</t>
-        </is>
-      </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
-        </is>
-      </c>
-      <c r="E101" s="5" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F101" s="5" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G101" s="5" t="inlineStr"/>
-      <c r="H101" s="5" t="inlineStr"/>
-      <c r="I101" s="5" t="inlineStr"/>
-      <c r="J101" s="5" t="inlineStr"/>
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>CAM-Raum</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>Gefahrstoffentsorgung (IPA)</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>(1) Anmeldeformular Sonderabfälle ausfüllen (Anzahl / Art) → (2) Formular freitags an die Sonderabfall-Mailbox senden (Abholung dienstags) → (3) Etiketten bedrucken (IPA = halogenfreie Lösungsmittel) → (4) Kanister bekleben: UN-Nr. horizontal, Gefahrstoffkleber Spitze nach oben → (5) Kanister in Gefahrstoffcontainer OS8/LFB (Pfortenschlüssel im Sekretariat) → (6) Leere Kanister: ausdampfen, Symbol durchstreichen, ohne Deckel in gelben Sack</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr"/>
+      <c r="H101" s="3" t="inlineStr"/>
+      <c r="I101" s="3" t="inlineStr"/>
+      <c r="J101" s="3" t="inlineStr"/>
     </row>
     <row r="102" ht="60" customHeight="1">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Intraoralscanner (IOS) Einweisung</t>
+          <t>IT / Software</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -4143,17 +4119,17 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
+          <t>(1) PC neu starten → (2) An-/Abmeldung und Netzwerkverbindung prüfen → (3) Hält das Problem an → IT-Service Tal</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr"/>
@@ -4164,32 +4140,32 @@
     <row r="103" ht="60" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Design-Prozess 4./5. Fachsemester</t>
+          <t>Unfall / Notfall</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
+          <t>(1) ⚠ Bei Verletzungen: Ärzte im Haus rufen, bei Bedarf Notarzt. SOP Unfallanzeige UKT beachten. Vorgesetzten informieren. Auge sofort an der Augendusche spülen, dabei aufhalten. Danach Arzt aufsuchen. Feuerlöscher: 1× Schaum. CO₂ bei Elektronik- und Flüssigkeitsbränden. Fluchtwege freihalten.</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>Zahnärztlicher Kollege</t>
+          <t>Sofortmaßnahme</t>
         </is>
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>Zuständigen zahnärztlichen Kollegen ansprechen</t>
+          <t>Ärzte im Haus rufen, bei Bedarf Notarzt | SOP Unfallanzeige UKT beachten</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr"/>
@@ -4200,12 +4176,12 @@
     <row r="104" ht="60" customHeight="1">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Schulungsvideos / Kompetenzmatrix</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -4215,17 +4191,17 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>(1) Auf ILIAS nach Schulungsvideos &amp; Kompetenzmatrix suchen → (2) Vor Gerätenutzung relevante Videos ansehen</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr"/>
@@ -4236,32 +4212,32 @@
     <row r="105" ht="60" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Slicing / Nesting für Kurse</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr"/>
@@ -4270,76 +4246,76 @@
       <c r="J105" s="3" t="inlineStr"/>
     </row>
     <row r="106" ht="60" customHeight="1">
-      <c r="A106" s="4" t="inlineStr">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>LEAN · 3D-Druck · KANBAN</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>3D-Druck-Anfrage stellen</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>(1) STL-Datei vorbereiten (geschlossenes Volumen, korrekte Größe) → (2) Kurze Beschreibung + gewünschtes Material angeben → (3) An die 3D-Druck-Mailbox senden</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>3D-Druck Mailbox</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr"/>
+      <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107" ht="60" customHeight="1">
+      <c r="A107" s="5" t="inlineStr">
         <is>
           <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
-      <c r="B106" s="4" t="inlineStr">
-        <is>
-          <t>Medientechnik</t>
-        </is>
-      </c>
-      <c r="C106" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D106" s="4" t="inlineStr">
-        <is>
-          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen → (2) Ohne Einweisung das Medienpanel nicht selbstständig bedienen</t>
-        </is>
-      </c>
-      <c r="E106" s="4" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>CAD/CAM Sicherheitseinweisung</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
+        <is>
+          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
+        </is>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
         <is>
           <t>Einweisung anfordern</t>
         </is>
       </c>
-      <c r="F106" s="4" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G106" s="4" t="inlineStr"/>
-      <c r="H106" s="4" t="inlineStr"/>
-      <c r="I106" s="4" t="inlineStr"/>
-      <c r="J106" s="4" t="inlineStr"/>
-    </row>
-    <row r="107" ht="60" customHeight="1">
-      <c r="A107" s="3" t="inlineStr">
-        <is>
-          <t>Qualifizierung · Einweisung</t>
-        </is>
-      </c>
-      <c r="B107" s="3" t="inlineStr">
-        <is>
-          <t>Haptic Device / 3D-Eingabestift</t>
-        </is>
-      </c>
-      <c r="C107" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="E107" s="3" t="inlineStr">
-        <is>
-          <t>Einweisung erforderlich</t>
-        </is>
-      </c>
-      <c r="F107" s="3" t="inlineStr">
-        <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G107" s="3" t="inlineStr"/>
-      <c r="H107" s="3" t="inlineStr"/>
-      <c r="I107" s="3" t="inlineStr"/>
-      <c r="J107" s="3" t="inlineStr"/>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G107" s="5" t="inlineStr"/>
+      <c r="H107" s="5" t="inlineStr"/>
+      <c r="I107" s="5" t="inlineStr"/>
+      <c r="J107" s="5" t="inlineStr"/>
     </row>
     <row r="108" ht="60" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
@@ -4349,7 +4325,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Einweisung KanbanSlides Excel</t>
+          <t>Intraoralscanner (IOS) Einweisung</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -4359,17 +4335,17 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
+          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr"/>
@@ -4385,7 +4361,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>KANBAN Materialverwaltung</t>
+          <t>Design-Prozess 4./5. Fachsemester</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -4395,17 +4371,17 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
+          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Zuständigen Kollegen ansprechen</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr"/>
@@ -4414,122 +4390,106 @@
       <c r="J109" s="3" t="inlineStr"/>
     </row>
     <row r="110" ht="60" customHeight="1">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Gebäude &amp; Infrastruktur</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>Wasser</t>
-        </is>
-      </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Hauptabsperrventil schließen, Bereich sichern. → (2) Betroffenen Bereich / Raum notieren. → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Sofort melden – alle Stellen erreichbar</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>Zuständige Stellen</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
-      <c r="I110" s="2" t="inlineStr"/>
-      <c r="J110" s="2" t="inlineStr"/>
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>Qualifizierung · Einweisung</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Schulungsvideos / Kompetenzmatrix</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>(1) Einführung in Adobe Premier Pro  (2) Einweisung in die Nutzung des Gimbals und de rAnsteckmikrofone</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>siehe Kompetenzmatrix</t>
+        </is>
+      </c>
+      <c r="G110" s="4" t="inlineStr"/>
+      <c r="H110" s="4" t="inlineStr"/>
+      <c r="I110" s="4" t="inlineStr"/>
+      <c r="J110" s="4" t="inlineStr"/>
     </row>
     <row r="111" ht="60" customHeight="1">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Gebäude &amp; Infrastruktur</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Strom / Elektrik</t>
+          <t>Slicing / Nesting für Kurse</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Geräte ausschalten, Bereich verlassen wenn nötig. → (2) Sicherungskasten prüfen – ist eine Sicherung ausgelöst? → (3) Betroffenen Bereich / Gerät notieren. → (4) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>Sofort melden – alle Stellen erreichbar</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
-      <c r="G111" s="3" t="inlineStr">
-        <is>
-          <t>Zuständige Stellen</t>
-        </is>
-      </c>
-      <c r="H111" s="3" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr"/>
+      <c r="H111" s="3" t="inlineStr"/>
       <c r="I111" s="3" t="inlineStr"/>
       <c r="J111" s="3" t="inlineStr"/>
     </row>
     <row r="112" ht="60" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>Gebäude &amp; Infrastruktur</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Klimatisierung / Lüftung</t>
+          <t>Medientechnik</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>(1) Betroffenen Raum und Art der Störung notieren (keine Kühlung, kein Luftstrom, Lärm, …). → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Stellen</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G112" s="4" t="inlineStr"/>
@@ -4540,76 +4500,68 @@
     <row r="113" ht="60" customHeight="1">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>Gebäude &amp; Infrastruktur</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Aufzug</t>
+          <t>Haptic Device / 3D-Eingabestift</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D113" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Ruhe bewahren – Person beruhigen, Notruf im Aufzug betätigen. → (2) Aufzug außer Betrieb kennzeichnen (Hinweis an der Tür). → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>Sofort melden – alle Stellen erreichbar</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>Notrufknopf im Aufzug betätigen (direkte Verbindung zur Aufzugswartung) | TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen | Notruf 112 wenn keine andere Hilfe erreichbar</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr">
-        <is>
-          <t>Zuständige Stellen</t>
-        </is>
-      </c>
-      <c r="H113" s="3" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
+          <t>Arzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr"/>
+      <c r="H113" s="3" t="inlineStr"/>
       <c r="I113" s="3" t="inlineStr"/>
       <c r="J113" s="3" t="inlineStr"/>
     </row>
     <row r="114" ht="60" customHeight="1">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Gebäude &amp; Infrastruktur</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Allgemeiner Defekt (Tür, Schloss, Mobiliar …)</t>
+          <t>Einweisung KanbanSlides Excel</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>(1) Defekt und genauen Ort (Raum, Tür, Möbel) kurz notieren. → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Stellen</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G114" s="4" t="inlineStr"/>
@@ -4620,27 +4572,27 @@
     <row r="115" ht="60" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Gebäude &amp; Infrastruktur</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Britta Wasserspender</t>
+          <t>KANBAN Materialverwaltung</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät ausschalten. → (2) Art der Störung notieren (kein Wasser, Filterwechsel fällig, Leck, ...). → (3) Technischen Koordinator oder Sekretariat informieren.</t>
+          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
@@ -4654,48 +4606,40 @@
       <c r="J115" s="3" t="inlineStr"/>
     </row>
     <row r="116" ht="60" customHeight="1">
-      <c r="A116" s="4" t="inlineStr">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>Gebäude &amp; Infrastruktur</t>
         </is>
       </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>Brandschutztür</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Wasser</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Brandschutztür nicht blockieren – Fluchtweg und Brandabschnitt müssen frei bleiben. → (2) Art des Problems notieren (schließt nicht vollständig, Geräusch, beschädigt, ...). → (3) TBA oder Werkstatt ZMK informieren.</t>
-        </is>
-      </c>
-      <c r="E116" s="4" t="inlineStr">
-        <is>
-          <t>Sofort melden</t>
-        </is>
-      </c>
-      <c r="F116" s="4" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
-      <c r="G116" s="4" t="inlineStr">
-        <is>
-          <t>Zuständige Stellen</t>
-        </is>
-      </c>
-      <c r="H116" s="4" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum)</t>
-        </is>
-      </c>
-      <c r="I116" s="4" t="inlineStr"/>
-      <c r="J116" s="4" t="inlineStr"/>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Hauptabsperrventil schließen, Bereich sichern. → (2) Betroffenen Bereich / Raum notieren. → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr"/>
+      <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
     </row>
     <row r="117" ht="60" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
@@ -4705,39 +4649,31 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Primion Schließsystem (Kartenzugang)</t>
+          <t>Strom / Elektrik</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>(1) Betroffenen Raum und Art des Defekts notieren. → (2) TBA oder IT-Service informieren.</t>
+          <t>(1) ⚠ Geräte ausschalten, Bereich verlassen wenn nötig. → (2) Sicherungskasten prüfen – ist eine Sicherung ausgelöst? → (3) Betroffenen Bereich / Gerät notieren. → (4) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="G117" s="3" t="inlineStr">
-        <is>
-          <t>Zuständige Stellen</t>
-        </is>
-      </c>
-      <c r="H117" s="3" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | IT-Service Tal – Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr"/>
+      <c r="H117" s="3" t="inlineStr"/>
       <c r="I117" s="3" t="inlineStr"/>
       <c r="J117" s="3" t="inlineStr"/>
     </row>
@@ -4749,27 +4685,27 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Flur E6 · Monitor – kein Bild</t>
+          <t>Klimatisierung / Lüftung</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>(1) Monitor eingeschaltet? → (2) Strom- und HDMI-Kabel geprüft?</t>
+          <t>(1) Betroffenen Raum und Art der Störung notieren (keine Kühlung, kein Luftstrom, Lärm, …). → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Stellen</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
         </is>
       </c>
       <c r="G118" s="4" t="inlineStr"/>
@@ -4785,33 +4721,249 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Flur E6 · Kalender wird nicht angezeigt</t>
+          <t>Aufzug</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>(1) Bitte melden!</t>
+          <t>(1) ⚠ Ruhe bewahren – Person beruhigen, Notruf im Aufzug betätigen. → (2) Aufzug außer Betrieb kennzeichnen (Hinweis an der Tür). → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Notrufknopf im Aufzug betätigen (direkte Verbindung zur Aufzugswartung) | TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen | Notruf 112 wenn keine andere Hilfe erreichbar</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr"/>
       <c r="H119" s="3" t="inlineStr"/>
       <c r="I119" s="3" t="inlineStr"/>
       <c r="J119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120" ht="60" customHeight="1">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>Allgemeiner Defekt (Tür, Schloss, Mobiliar …)</t>
+        </is>
+      </c>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>(1) Defekt und genauen Ort (Raum, Tür, Möbel) kurz notieren. → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Zuständige Stellen</t>
+        </is>
+      </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="inlineStr"/>
+      <c r="H120" s="4" t="inlineStr"/>
+      <c r="I120" s="4" t="inlineStr"/>
+      <c r="J120" s="4" t="inlineStr"/>
+    </row>
+    <row r="121" ht="60" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Britta Wasserspender</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>(1) Gerät ausschalten. → (2) Art der Störung notieren (kein Wasser, Filterwechsel fällig, Leck, ...). → (3) Technischen Koordinator oder Sekretariat informieren.</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr"/>
+      <c r="H121" s="3" t="inlineStr"/>
+      <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122" ht="60" customHeight="1">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Brandschutztür</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Brandschutztür nicht blockieren – Fluchtweg und Brandabschnitt müssen frei bleiben. → (2) Art des Problems notieren (schließt nicht vollständig, Geräusch, beschädigt, ...). → (3) TBA oder Werkstatt ZMK informieren.</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr"/>
+      <c r="H122" s="4" t="inlineStr"/>
+      <c r="I122" s="4" t="inlineStr"/>
+      <c r="J122" s="4" t="inlineStr"/>
+    </row>
+    <row r="123" ht="60" customHeight="1">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Primion Schließsystem (Kartenzugang)</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>(1) Betroffenen Raum und Art des Defekts notieren. → (2) TBA oder IT-Service informieren.</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr"/>
+      <c r="H123" s="3" t="inlineStr"/>
+      <c r="I123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124" ht="60" customHeight="1">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Flur E6 · Monitor – kein Bild</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>(1) Monitor eingeschaltet? → (2) Strom- und HDMI-Kabel geprüft?</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G124" s="4" t="inlineStr"/>
+      <c r="H124" s="4" t="inlineStr"/>
+      <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125" ht="60" customHeight="1">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Flur E6 · Kalender wird nicht angezeigt</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>(1) Bitte melden!</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr"/>
+      <c r="H125" s="3" t="inlineStr"/>
+      <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>

</xml_diff>

<commit_message>
Add dual-contact boxes to Ansprechpartner view + apply updated Excel
UI: when Ansprechpartner finden is pressed, show 1. and 2. Ansprechpartner
side-by-side in small boxes; contact details render below both boxes.

Data: re-apply all 122 rows from reviewed Excel (a49d8529) —
19 contact/step corrections, 2 new devices (Erkoform 3d motion
(Tiefziehgerät), Phantomkopf & Torso), 5 deletions (Medienpanel
Extron, Kamera/Medientechnik defekt, Demokamera, Notschalter,
old Erkoform). AP2 (col G/H) now stored as ap2:{name,lines} in
every contact/escalation node (80 devices total).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019KwCcZLvcVY13HRSnpAd9T
</commit_message>
<xml_diff>
--- a/Ansprechpartner_Review.xlsx
+++ b/Ansprechpartner_Review.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -712,7 +712,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Medienpanel (Extron)</t>
+          <t>Beamer Seminarraum</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -779,17 +779,17 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>(1) Medienpanel in SR1 &amp; SR2 ausschalten, dann in SR1 einschalten (ca. 90 Sekunden) → (2) Cave: Nach Benutzung immer ausschalten.</t>
+          <t>(1) Ist der Projektor am Medienpanel eingeschaltet? → (2) Ist Bild Aus/Ein aktiviert (rot oder grün)? → (3) Ist die Bildquelle korrekt ausgewählt? (4) Windowstaste+P klickenauf Account clicken und Dublizieren/Erweitern auswählen</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Assistenzarzt Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
@@ -805,7 +805,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Beamer Seminarraum</t>
+          <t>Klimatisierung</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -815,17 +815,17 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>(1) Ist der Projektor am Medienpanel eingeschaltet? → (2) Ist Bild Aus/Ein aktiviert (rot oder grün)? → (3) Ist die Bildquelle korrekt ausgewählt? (4) Windowstaste+P klickenauf Account clicken und Dublizieren/Erweitern auswählen</t>
+          <t>(1) Die Klimaanlage lässt sich über den Regler neben der Tür regeln. → (2) Die Mittelstellung entspricht 24 °C. → (3) Schneemann: 21 °C. → (4) Sonne: 27 °C. → (5) Die Regelung der Raumtemperatur erfolgt nur bei geschlossenen Fenstern &amp; Tür. → (6) Nach der automatischen Abschaltung der Anlage um 16:30 (Mond), lässt sich diese durch Drücken des Männchen wieder aktivieren.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr"/>
@@ -841,27 +841,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Klimatisierung</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>(1) Die Klimaanlage lässt sich über den Regler neben der Tür regeln. → (2) Die Mittelstellung entspricht 24 °C. → (3) Schneemann: 21 °C. → (4) Sonne: 27 °C. → (5) Die Regelung der Raumtemperatur erfolgt nur bei geschlossenen Fenstern &amp; Tür. → (6) Nach der automatischen Abschaltung der Anlage um 16:30 (Mond), lässt sich diese durch Drücken des Männchen wieder aktivieren.</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
@@ -870,76 +870,76 @@
       <c r="J10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Seminar 1</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>PC / Workstation – Funktionsstörung</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Seminar 2</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Trennwände – Räume kombinieren/teilen</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Die Kurbel liegt für gewöhnlich in einem der Medienkoffer in SR1 oder SR3. → (2) Erklärvideo auf Q:\</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Seminar 2</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Trennwände – Räume kombinieren/teilen</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Die Kurbel liegt für gewöhnlich in einem der Medienkoffer in SR1 oder SR3. → (2) Erklärvideo auf Q:\</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Buchung / Zugang</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Ausstattung – Lautsprecher</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -959,91 +959,91 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Seminar 2 ist analog ausgestattet: Metaplan-Wand und Flipchart. Keine fest installierte AV-Technik. → (2) In diesem Raum befindet sich ein zusätzlicher Lautsprecher, welcher sich vom Medienpanel SR3 steuern lässt.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
-        </is>
-      </c>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
       <c r="G13" s="3" t="inlineStr"/>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Seminar 2</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Ausstattung – Lautsprecher</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>(1) Seminar 2 ist analog ausgestattet: Metaplan-Wand und Flipchart. Keine fest installierte AV-Technik. → (2) In diesem Raum befindet sich ein zusätzlicher Lautsprecher, welcher sich vom Medienpanel SR3 steuern lässt.</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>AV-Medien</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
-      <c r="I14" s="4" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Seminar 3</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Medienpanel / Raumsteuerung</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>(1) Medienpanel in SR1 &amp; SR3 ausschalten, dann in SR1 einschalten (ca. 90 Sekunden) → (2) Cave: Nach Benutzung immer ausschalten.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Seminar 3</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Medienpanel / Raumsteuerung</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>(1) Medienpanel in SR1 &amp; SR3 ausschalten, dann in SR1 einschalten (ca. 90 Sekunden) → (2) Cave: Nach Benutzung immer ausschalten.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>ClickShare</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>(1) ClickShare in den USB-Eingang vom Laptop einstecken → (2) ClickShare wie USB-Stick im Explorer öffnen und die Windows-App starten → (3) Bildschirm freigeben (App oder Button drücken) → (4) Kein Bild? App schließen, neu starten, erneut verbinden, USB wechseln → (5) Ist die richtige Quelle auf dem Medienpanel ausgewählt?</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>IT-Service Tal</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>ClickShare</t>
+          <t>Mikrofon (drahtlos)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1063,12 +1063,12 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>(1) ClickShare in den USB-Eingang vom Laptop einstecken → (2) ClickShare wie USB-Stick im Explorer öffnen und die Windows-App starten → (3) Bildschirm freigeben (App oder Button drücken) → (4) Kein Bild? App schließen, neu starten, erneut verbinden, USB wechseln → (5) Ist die richtige Quelle auf dem Medienpanel ausgewählt?</t>
+          <t>(1) Akku prüfen – ist das Mikrofon geladen? → (2) Empfänger eingeschaltet? → (3) Richtiger Eingang am Medienpanel ausgewählt? → (4) Lautstärke am Panel aufgedreht? → (5) Wenn Mikro nicht reagiert, aufschrauben und die Batterie neu einsetzen.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Mikrofon (drahtlos)</t>
+          <t>KI-Tracking-Kamera</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>(1) Akku prüfen – ist das Mikrofon geladen? → (2) Empfänger eingeschaltet? → (3) Richtiger Eingang am Medienpanel ausgewählt? → (4) Lautstärke am Panel aufgedreht? → (5) Wenn Mikro nicht reagiert, aufschrauben und die Batterie neu einsetzen.</t>
+          <t>(1) Steuerung erfolgt über den Button "360° Kamera" auf dem Medienpanel. → (2) Es muss die richtige Quelle unter Projektion ausgewählt sein.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr"/>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>KI-Tracking-Kamera</t>
+          <t>Patientenkamera</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1135,17 +1135,17 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>(1) Steuerung erfolgt über den Button "360° Kamera" auf dem Medienpanel. → (2) Es muss die richtige Quelle unter Projektion ausgewählt sein.</t>
+          <t>(1) Akkus liegen auf Dozenten PC in SR 1 und sollten nach Benutzung dort geladen werden. → (2) Akku in die Kamera einsetzen und Kamera seitlich einschalten. → (3) Signal über das Medienpanel richtig zuweisen.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>AV-Medien</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Patientenkamera</t>
+          <t>Aufnahme über AV-Netz</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1171,17 +1171,17 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>(1) Akkus liegen auf Dozenten PC in SR 1 und sollten nach Benutzung dort geladen werden. → (2) Akku in die Kamera einsetzen und Kamera seitlich einschalten. → (3) Signal über das Medienpanel richtig zuweisen.</t>
+          <t>(1) Seminar 3 ist über das AV-Netz zur Aufnahme angebunden. Aufnahme über das Medienpanel starten.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Arzt Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Aufnahme über AV-Netz</t>
+          <t>Trennwände – Räume kombinieren/teilen</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1207,19 +1207,15 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>(1) Seminar 3 ist über das AV-Netz zur Aufnahme angebunden. Aufnahme über das Medienpanel starten.</t>
+          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Erklärvideo auf Q:\</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>AV-Medien</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
           <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
+      <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr"/>
@@ -1233,7 +1229,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Trennwände – Räume kombinieren/teilen</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1243,15 +1239,19 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>(1) Die Seminarräume 1, 2 und 3 lassen sich über die Trennwände zu einem großen Raum verbinden oder einzeln nutzen. Erklärvideo auf Q:\</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+        </is>
+      </c>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
@@ -1265,27 +1265,27 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Kamera / Medientechnik defekt</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät über das Medienpanel kurz aus- und wieder einschalten → (2) Kabel- und Signalverbindung am Panel prüfen</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>AV-Medien</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Mit Einweisung → direkt kontaktieren | Ohne Einweisung → zuerst Techn. Koordinator</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr"/>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Patientenkamera /</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1311,17 +1311,17 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Gerät über das Medienpanel kurz aus- und wieder einschalten → (2) Kabel- und Signalverbindung dewr Kamera prüfen</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Mit Einweisung → direkt kontaktieren | Ohne Einweisung → zuerst Techn. Koordinator</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr"/>
@@ -1330,50 +1330,50 @@
       <c r="J23" s="3" t="inlineStr"/>
     </row>
     <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Seminar 3</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>PC / Workstation – Funktionsstörung</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="4" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Technicum</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Hotty Wax Station</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>(1) Temperatur je nach Wachstyp einstellen – mind. 10 Min. vorheizen lassen. → (2) Nur zugelassene Dentalwachse verwenden. → (3) Instrumente im Gerät reinigen, bevor die Arbeit beginnt. → (4) Nach Gebrauch: Gerät ausschalten und reinigen.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Seminar 3</t>
+          <t>Technicum</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Patientenkamera /</t>
+          <t>Intraoralscanner</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1383,17 +1383,17 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät über das Medienpanel kurz aus- und wieder einschalten → (2) Kabel- und Signalverbindung dewr Kamera prüfen</t>
+          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>AV-Medien</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Mit Einweisung → direkt kontaktieren | Ohne Einweisung → zuerst Techn. Koordinator</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr"/>
@@ -1402,40 +1402,40 @@
       <c r="J25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="60" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Technicum</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Hotty Wax Station</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>(1) Temperatur je nach Wachstyp einstellen – mind. 10 Min. vorheizen lassen. → (2) Nur zugelassene Dentalwachse verwenden. → (3) Instrumente im Gerät reinigen, bevor die Arbeit beginnt. → (4) Nach Gebrauch: Gerät ausschalten, keine Wachsreste im Becken lassen.</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Sirona SIM Intego Bench</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>(1) Fußschalter prüfen – eingesteckt und im richtigen Modus? → (2) Handstück einsetzen bis es hörbar einrastet. → (3) Wasser  kommt nicht?  Drehregler am Motor öffnen (3.1) Luft kommt nicht -&gt; Aufsatz auf verstopfung prüfen→ (4) Licht am Winkelstück geht nicht? fest einstecken und Knopf an der Einheit an? → (4) Gerät reagiert gar nicht? Hauptschalter prüfen.</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -1445,27 +1445,23 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Intraoralscanner</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr"/>
@@ -1481,17 +1477,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Sirona SIM Intego Bench</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>(1) Fußschalter prüfen – eingesteckt und im richtigen Modus? → (2) Handstück einsetzen bis es hörbar einrastet. → (3) Wasser / Luft kommt nicht? Absperrventil am Gerät öffnen. → (4) Licht defekt? Handstücklampe prüfen (fest einschrauben). → (5) Gerät reagiert gar nicht? Hauptschalter an der Rückseite prüfen.</t>
+          <t>(1) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (2) Knopf am System 3 Sekunden gedrückt halten</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1501,7 +1497,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr"/>
@@ -1517,23 +1513,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Medienpanel / Raumsteuerung</t>
+          <t>Noflame Plus</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr"/>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>(1) Instrument aus der Spulenöffnung nehmen → (2) Gerät aus- und wieder einschalten → (3) Lüftungsschlitze freiräumen → (4) Gerät ausschalten → (5) Einige Minuten abkühlen lassen → (6) Neu starten</t>
+        </is>
+      </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
@@ -1549,17 +1549,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>QUATTROcare</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
+          <t>(1) Ersatzkartuschen bei den Aufsichten. Kartuschen können selbst gewechselt werden.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr"/>
@@ -1585,27 +1585,27 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Noflame Plus</t>
+          <t>Bildschirme schwarz</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>(1) Instrument aus der Spulenöffnung nehmen → (2) Gerät aus- und wieder einschalten → (3) Lüftungsschlitze freiräumen → (4) Gerät ausschalten → (5) Einige Minuten abkühlen lassen → (6) Neu starten</t>
+          <t>(1) Am Medienpanel richtiges Signal ausgewählt? → (2) Signal neu zuweisen. → (3) Bildschirm am Panel aus- und wieder einschalten</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr"/>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>QUATTROcare</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>(1) Ersatzkartuschen bei den Aufsichten. Kartuschen können selbst gewechselt werden.</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
@@ -1657,7 +1657,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Demokamera</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1667,17 +1667,17 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC auf Input 1 zurückschalten -</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Einweisung erforderlich</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Assistenzarzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr"/>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Bildschirme schwarz</t>
+          <t>Präpchecker / Dental Teacher</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -1703,17 +1703,17 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>(1) Am Medienpanel richtiges Signal ausgewählt? → (2) Signal neu zuweisen. → (3) Bildschirm am Panel aus- und wieder einschalten</t>
+          <t>(1) Demopräps sind hinterlegt. → (2) Einweisung durch Kurs</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr"/>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Notschalter ausgelöst</t>
+          <t>Pentamix 3</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>(1) Prüfen ob der Auslösegrund behoben ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
+          <t>(1) Bedienung im Kurs nach Einführung selbstständig.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr"/>
@@ -1765,19 +1765,15 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>Mikroskop (Leica A60)</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
-        </is>
-      </c>
+          <t>contact</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
@@ -1785,7 +1781,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Arzt im Raum „Besprechung Lehrende“ ansprechen</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
@@ -1801,27 +1797,27 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender/Moses Med prüfen → (2) Freien Termin anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr"/>
@@ -1837,7 +1833,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Präpchecker / Dental Teacher</t>
+          <t>Labcam / Demokamera</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -1847,17 +1843,17 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>(1) Demopräps sind hinterlegt. → (2) Einweisung durch Kurs</t>
+          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC, Switch auf Input 1 schalten.-</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>AV-Medien</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr"/>
@@ -1873,15 +1869,19 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Pentamix 3</t>
+          <t>Kein Strom an allen Plätzen</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>contact</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>(1) Prüfen obNotschalter ausgelöst ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr"/>
@@ -1905,15 +1905,19 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Mikroskop (Leica A60)</t>
+          <t>Handstück dreht links</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>contact</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>(1) Fehler F5: Kniesteuerung komplett ausschalten (10s warten) → (2) Linkslauf: Gerät ist im Linksbetrieb! → (3) Am Netzschalter (11) ausschalten → (4) Rechtslauftaste T4 (Plustaste) gedrückt halten → (5) Dabei Netzschalter wieder einschalten → (6) LED T3 aus = Rechtslauf aktiv</t>
+        </is>
+      </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
@@ -1921,7 +1925,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Arzt im Raum „Besprechung Lehrende“ ansprechen</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
@@ -1930,50 +1934,50 @@
       <c r="J40" s="4" t="inlineStr"/>
     </row>
     <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Technicum</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>PC / Workstation – Funktionsstörung</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr"/>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Phantomicum</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Arbeitsplatzkamera</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>(1) Richtige Kameraquelle am Panel ausgewählt (2) NDI-PC gestartet? → (2) Notschalter an?</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>AV-Medien</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="5" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Technicum</t>
+          <t>Phantomicum</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Labcam / Demokamera</t>
+          <t>Intraoralscanner</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -1983,17 +1987,17 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>(1) Kamerasteuermodul eingeschaltet? (silberne Box - Firma RIETH.) → (2) Schutzdeckel von der Kamera entfernt? → (3) Signal am Medienpanel korrekt zugewiesen? → (4) Bild nur auf dem Bildschirm angezeigt? Switch unter dem Tisch rechts auf Input 2 schalten. → (5) - Für Dozenten PC, Switch auf Input 1 schalten.-</t>
+          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>AV-Medien</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: AV-Medien</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr"/>
@@ -2004,12 +2008,12 @@
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Technicum</t>
+          <t>Phantomicum</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Kein Strom an allen Plätzen</t>
+          <t>Pentamix 3</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2019,7 +2023,7 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>(1) Prüfen ob der Auslösegrund behoben ist → (2) Notschalter wieder eindrücken / zurücksetzen → (3) Geräte neu starten</t>
+          <t>(1) Bedienung im Kurs nach Einführung selbstständig.</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
@@ -2029,7 +2033,7 @@
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr"/>
@@ -2040,32 +2044,28 @@
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Technicum</t>
+          <t>Phantomicum</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Handstück dreht links</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>(1) Fehler F5: Kniesteuerung komplett ausschalten (10s warten) → (2) Linkslauf: Gerät ist im Linksbetrieb! → (3) Am Netzschalter (11) ausschalten → (4) Rechtslauftaste T4 (Plustaste) gedrückt halten → (5) Dabei Netzschalter wieder einschalten → (6) LED T3 aus = Rechtslauf aktiv</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr"/>
@@ -2074,40 +2074,40 @@
       <c r="J44" s="4" t="inlineStr"/>
     </row>
     <row r="45" ht="60" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>Phantomicum</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>Arbeitsplatzkamera</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>(1) Richtige Kameraquelle am Panel ausgewählt (2) NDI-PC gestartet? → (2) Notschalter an?</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>AV-Medien</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr"/>
-      <c r="H45" s="5" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="5" t="inlineStr"/>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Behandlungseinheit / Turbine / Handstück</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>(1) Bei wasseraustritt am Schlauch, ausschalten und sofort die Werkstatt rufen! (1) Ist die Behandlungseinheit eingeschaltet? → (2) Handstück/Turbine korrekt aufgesteckt und eingerastet? → (3) Einheit kurz aus- und wieder einschalten → (4) Helligkeit am Bedienfeld geprüft?  (9) Fußanlasser betätigt? → (5) Schläuche nicht geknickt?</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Intraoralscanner</t>
+          <t>QUATTROcare</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2127,7 +2127,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>(1) Nur während aktiver Nutzung im Raum verfügbar. → (2) Bedienung nach IOS-Einweisung – Gebrauchsanweisung beachten.</t>
+          <t>(1) Ersatzkartuschen bei den Aufsichten. Handstückpflege durch Studierende selbst.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Pentamix 3</t>
+          <t>Cavex Alginate Mixer</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>(1) Bedienung im Kurs nach Einführung selbstständig.</t>
+          <t>(1) Bedienung im Kurs nach Einführung durch Aufsichten selbstständig.</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr"/>
@@ -2189,23 +2189,27 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Medienpanel / Raumsteuerung</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+        </is>
+      </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
@@ -2221,27 +2225,27 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Behandlungseinheit / Turbine / Handstück</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>(1) Ist die Behandlungseinheit eingeschaltet? → (2) Druckluft- und Wasser-Haupthahn geöffnet? → (3) Handstück/Turbine korrekt aufgesteckt und eingerastet? → (4) Einheit kurz aus- und wieder einschalten → (5) Lichtschalter an der Einheit betätigt? → (6) Helligkeit am Bedienfeld geprüft? → (7) Einheit aus- und wieder einschalten → (8) Haupthahn für Wasser und Druckluft geöffnet? → (9) Fußanlasser betätigt? → (10) Schläuche korrekt angeschlossen und nicht geknickt?</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr"/>
@@ -2257,7 +2261,7 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>QUATTROcare</t>
+          <t>Phantomkopf &amp; Torso (SIM-Einheit)</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -2267,7 +2271,7 @@
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>(1) Ersatzkartuschen bei den Aufsichten. Handstückpflege durch Studierende selbst.</t>
+          <t>(1) Nur nach lösen der Befestigungsschraube das Kugelgelenk bewegen!</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
@@ -2277,7 +2281,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Sekretariat / Koordination Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
@@ -2286,50 +2290,50 @@
       <c r="J50" s="4" t="inlineStr"/>
     </row>
     <row r="51" ht="60" customHeight="1">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>Phantomicum</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>Cavex Alginate Mixer</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>(1) Bedienung im Kurs nach Einführung durch Aufsichten selbstständig.</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Gipsen &amp; Polieren</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Absaugbox BIOSTEAM Center</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>(1) Hauptschalter drücken – Gerät läuft, sobald Absaugung aktiv ist (hörbar). → (2) Schlauch auf Knickstellen oder Verstopfungen prüfen. → (3) Saugleistung schwach? Filter / Sieb prüfen und ggf. reinigen. → (4) Wasserbehälter entleeren wenn Füllstand-Anzeige leuchtet.</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr"/>
-      <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="3" t="inlineStr"/>
-      <c r="J51" s="3" t="inlineStr"/>
+      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Phantomicum</t>
+          <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Steamy Mini (Abdampfer)</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -2339,17 +2343,17 @@
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) Wassertank befüllen (destilliertes Wasser – nur bei abgekühltem Gerät). → (2) Aufheizzeit abwarten – ca. 3–5 Min. bis Betriebsdruck erreicht ist. → (3) Nach Gebrauch: Ausschalten, Restdampf ablassen.</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
@@ -2360,32 +2364,32 @@
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>Phantomicum</t>
+          <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>PC / Workstation – Funktionsstörung</t>
+          <t>Trockentrimmer</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Hauptschalter prüfen – Absaugung muss laufen (hörbar), erst dann trimmen. → (2) Modell flach und gerade aufsetzen, gleichmäßigen Druck ausüben – nicht verkanten. → (3) Sollte das Schleifband verrutscht sein, bitte nicht selbst reparieren.</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr"/>
@@ -2394,40 +2398,40 @@
       <c r="J53" s="3" t="inlineStr"/>
     </row>
     <row r="54" ht="60" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>Gipsen &amp; Polieren</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Absaugbox BIOSTEAM Center</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>(1) Hauptschalter drücken – Gerät läuft, sobald Absaugung aktiv ist (hörbar). → (2) Schlauch auf Knickstellen oder Verstopfungen prüfen. → (3) Saugleistung schwach? Filter / Sieb prüfen und ggf. reinigen. → (4) Wasserbehälter entleeren wenn Füllstand-Anzeige leuchtet.</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Giroform</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>(1) Nur nach erfolgter Einweisung verwenden. → (2) Stiftposition nach Kursanleitung wählen – Stifte korrekt einsetzen und sichern. → (3) Modell in Artikulator einsetzen: Index-Stifte korrekt ausrichten und einrasten lassen.</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr"/>
+      <c r="H54" s="4" t="inlineStr"/>
+      <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr"/>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
@@ -2437,7 +2441,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Steamy Mini (Abdampfer)</t>
+          <t>Smartbox X2</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -2447,7 +2451,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>(1) Wassertank befüllen (destilliertes Wasser – nur bei abgekühltem Gerät). → (2) Aufheizzeit abwarten – ca. 3–5 Min. bis Betriebsdruck erreicht ist. → (3) Düse verstopft? Nadel aus dem Zubehör vorsichtig durchstecken. → (4) Nach Gebrauch: Ausschalten, Restdampf ablassen.</t>
+          <t>(1) Wasser einfüllen, Gerät einschalten – Vorheizzeit ca. 5 Min. abwarten. → (2) Küvette einlegen, Deckel fest verschließen – O-Ring auf Sauberkeit prüfen. → (3) Druck und Zeit gemäß Kursanleitung einstellen. → (4) Nach Ende: Druck über Ablassventil langsam ablassen, erst dann öffnen.</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
@@ -2473,7 +2477,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Trockentrimmer</t>
+          <t>Smartmix</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -2483,7 +2487,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>(1) Hauptschalter prüfen – Absaugung muss laufen (hörbar), erst dann trimmen. → (2) Modell flach und gerade aufsetzen, gleichmäßigen Druck ausüben – nicht verkanten. → (3) Sollte das Schleifband verrutscht sein, bitte nicht selbst reparieren.</t>
+          <t>(1) Schüssel und Paddel korrekt einsetzen und verriegeln. → (2) Wasser-Pulver-Verhältnis nach Anleitung abmessen (Messbecher verwenden). → (3) Mischzeit je nach Material einstellen (Gips ca. 30–45 s, Alginat ca. 45–60 s). → (4) Nach Gebrauch Schüssel und Paddel sofort reinigen.</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
@@ -2509,7 +2513,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Erkoform 3d motion</t>
+          <t>Polierbox</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2519,7 +2523,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>(1) Folientyp und -stärke laut Kursanleitung wählen (Aufkleber am Gerät beachten). → (2) Folie sorgfältig einspannen – Rahmen gleichmäßig und fest schließen. → (3) Temperatur und Druck je nach Material einstellen. → (4) Folie reißt? Temperatur oder Foliendicke prüfen, ggf. neu einspannen. → (5) Nach Abkühlung Modell entnehmen, Folie vorsichtig abtrennen.</t>
+          <t>(1) Absaugung einschalten – Schalter am Gerät oder Fußpedal prüfen. → (2) Drehzahl am Handstück je nach Werkstück wählen. → (3) Saugleistung schwach? Filterbeutel / Sieb prüfen und ggf. reinigen. → (4) Handstück und Schleifkörper nach Nutzung reinigen.</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -2545,17 +2549,17 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Giroform</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>(1) Nur nach erfolgter Einweisung verwenden. → (2) Stiftposition nach Kursanleitung wählen – Stifte korrekt einsetzen und sichern. → (3) Modell in Artikulator einsetzen: Index-Stifte korrekt ausrichten und einrasten lassen.</t>
+          <t>(1) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (2) Knopf am System 3 Sekunden gedrückt halten</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
@@ -2565,7 +2569,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr"/>
@@ -2581,7 +2585,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Smartbox X2</t>
+          <t>Abdampfgerät D-S100A</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2591,7 +2595,7 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>(1) Wasser einfüllen, Gerät einschalten – Vorheizzeit ca. 5 Min. abwarten. → (2) Küvette einlegen, Deckel fest verschließen – O-Ring auf Sauberkeit prüfen. → (3) Druck und Zeit gemäß Kursanleitung einstellen. → (4) Nach Ende: Druck über Ablassventil langsam ablassen, erst dann öffnen.</t>
+          <t>(1) Wasserhahn aufgedreht? → (2) Hauptschaulter am Gerät ein? (3) Aufgeheizt? (4) Fußschalter betätigen.</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
@@ -2617,7 +2621,7 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Smartmix</t>
+          <t>Gipstrimmer HSS-88</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -2627,7 +2631,7 @@
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>(1) Schüssel und Paddel korrekt einsetzen und verriegeln. → (2) Wasser-Pulver-Verhältnis nach Anleitung abmessen (Messbecher verwenden). → (3) Mischzeit je nach Material einstellen (Gips ca. 30–45 s, Alginat ca. 45–60 s). → (4) Nach Gebrauch Schüssel und Paddel sofort reinigen.</t>
+          <t>(1) Ist der Wasserhahn aufgedreht? !!!</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
@@ -2653,7 +2657,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Polierbox</t>
+          <t>Rüttler</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -2663,7 +2667,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>(1) Absaugung einschalten – Schalter am Gerät oder Fußpedal prüfen. → (2) Drehzahl am Handstück je nach Werkstück wählen. → (3) Saugleistung schwach? Filterbeutel / Sieb prüfen und ggf. reinigen. → (4) Handstück und Schleifkörper nach Nutzung reinigen.</t>
+          <t>(1) Ein/Aus-Schalter und Intensitätsregler prüfen.</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -2689,17 +2693,17 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>Elmasonic S (Ultraschall)</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
+          <t>(1) Wasser bis zur Markierung nachfüllen, dann neu starten.</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
@@ -2709,7 +2713,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr"/>
@@ -2725,7 +2729,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Abdampfgerät D-S100A</t>
+          <t>Erkoform 3d+</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2735,7 +2739,7 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>(1) Wasserhahn aufgedreht? → (2) Wasserstand im zweiten Abdampfer prüfen – ggf. nachfüllen</t>
+          <t>(1) Nur nach erfolgter Einweisung bedienen → (2) Folie und Einstellungen nach Kursanleitung wählen → (3) Bei Unsicherheit Einweisung anfordern</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
@@ -2761,7 +2765,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Gipstrimmer HSS-88</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -2771,7 +2775,7 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>(1) Ist der Wasserhahn aufgedreht? Das ist der häufigste Grund.</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
@@ -2781,7 +2785,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
@@ -2797,27 +2801,27 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Rüttler</t>
+          <t>Gipsabscheider</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>(1) Ein/Aus-Schalter und Intensitätsregler prüfen.</t>
+          <t>(1) Gerät nicht selbst öffnen oder entleeren. → (2) Füllstand / Störmeldung notieren.</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Für Lehrungen, Hauswirtschaft kontaktieren</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr"/>
@@ -2833,7 +2837,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Elmasonic S (Ultraschall)</t>
+          <t>Erkoform 3d motion (Tiefziehgerät)</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -2843,7 +2847,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>(1) Wasser bis zur Markierung nachfüllen, dann neu starten.</t>
+          <t>(1) Folientyp und -stärke laut Kursanleitung wählen (Aufkleber am Gerät beachten). → (2) Folie sorgfältig einspannen – Rahmen gleichmäßig und fest schließen. → (3) Temperatur und Druck je nach Material einstellen. → (4) Folie reißt? Temperatur oder Foliendicke prüfen, ggf. neu einspannen. → (5) Nach Abkühlung Modell entnehmen, Folie vorsichtig abtrennen.</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -2862,60 +2866,60 @@
       <c r="J66" s="4" t="inlineStr"/>
     </row>
     <row r="67" ht="60" customHeight="1">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>Gipsen &amp; Polieren</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>Erkoform 3d+</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>(1) Nur nach erfolgter Einweisung bedienen → (2) Folie und Einstellungen nach Kursanleitung wählen → (3) Bei Unsicherheit Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr"/>
-      <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="3" t="inlineStr"/>
-      <c r="J67" s="3" t="inlineStr"/>
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Gießen &amp; Strahlen</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Augenspülstation</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Bei Spritzern ins Auge sofort ausgiebig mit der Augenspülstation spülen (mind. 30 s) und Lehrpersonal informieren. → (2) Standort: im Raum Gießen &amp; Strahlen. Betroffenes Auge sofort und ausgiebig spülen, Augenlid offen halten. Anschließend Lehrpersonal informieren und – außer bei Bagatelle – Unfallmeldung ausfüllen. Station stets frei zugänglich halten; Verfallsdatum der Spülflaschen beachten. → (3) Keine Gewähr der Angaben</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="5" t="inlineStr"/>
+      <c r="I67" s="5" t="inlineStr"/>
+      <c r="J67" s="5" t="inlineStr"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>Gipsen &amp; Polieren</t>
+          <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>Trockenabsaugung</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
+          <t>(1) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (2) Knopf am System 3 Sekunden gedrückt halten</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -2925,7 +2929,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
@@ -2936,32 +2940,32 @@
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Gipsen &amp; Polieren</t>
+          <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Gipsabscheider</t>
+          <t>eyevolution max</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät nicht selbst öffnen oder entleeren. → (2) Füllstand / Störmeldung notieren.</t>
+          <t>(1) Ein/Aus-Schalter prüfen, Gerät neu starten. Am Strom angeschlossen? → (2) Programm nach Kursanleitung anpassen.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr.</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr"/>
@@ -2970,40 +2974,40 @@
       <c r="J69" s="3" t="inlineStr"/>
     </row>
     <row r="70" ht="60" customHeight="1">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>Gießen &amp; Strahlen</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Augenspülstation</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Bei Spritzern ins Auge sofort ausgiebig mit der Augenspülstation spülen (mind. 30 s) und Lehrpersonal informieren. → (2) Standort: im Raum Gießen &amp; Strahlen. Betroffenes Auge sofort und ausgiebig spülen, Augenlid offen halten. Anschließend Lehrpersonal informieren und – außer bei Bagatelle – Unfallmeldung ausfüllen. Station stets frei zugänglich halten; Verfallsdatum der Spülflaschen beachten. → (3) Keine Gewähr der Angaben</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr"/>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Sandstrahl BA9001</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>(1) Druckluftanschluss prüfen – ist der Hahn geöffnet? → (2) Korrekte Körnung beim Auffüllen verwendet? Sand nach Kursanleitung nachfüllen. → (3) Kabinenfenster von innen reinigen und neue Klarsichtfolie erneuert.</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
+      <c r="H70" s="4" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr"/>
     </row>
     <row r="71" ht="60" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
@@ -3013,17 +3017,17 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Trockenabsaugung</t>
+          <t>Drucktopf</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>(1) Schlauchverbindung am Arbeitsplatz prüfen – korrekt eingesteckt? → (2) System eingeschaltet? Das Einschalten erfolgt durch die Aufsicht im Raum „Besprechung Lehrende“. → (3) Knopf am System 3 Sekunden gedrückt halten → (4) Powermodus läuft 15 Minuten</t>
+          <t>(1) ⚠ Den Drucktopf niemals ohne Einweisung bedienen – immer erst Druck vollständig ablassen!</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -3033,7 +3037,7 @@
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Aufsicht / Arzt im Raum „Besprechung Lehrende“ ansprechen | Nur sie dürfen das System ein- und ausschalten</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr"/>
@@ -3049,7 +3053,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>eyevolution max</t>
+          <t>Gerät defekt melden</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -3059,7 +3063,7 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>(1) Ein/Aus-Schalter prüfen, Gerät neu starten. Am Strom angeschlossen? → (2) Programm nach Kursanleitung anpassen.</t>
+          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -3069,7 +3073,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
+          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr"/>
@@ -3078,72 +3082,68 @@
       <c r="J72" s="4" t="inlineStr"/>
     </row>
     <row r="73" ht="60" customHeight="1">
-      <c r="A73" s="3" t="inlineStr">
-        <is>
-          <t>Gießen &amp; Strahlen</t>
-        </is>
-      </c>
-      <c r="B73" s="3" t="inlineStr">
-        <is>
-          <t>Sandstrahl BA9001</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>(1) Druckluftanschluss prüfen – ist der Hahn geöffnet? → (2) Düse vorsichtig nach Kursanleitung reinigen. → (3) Sand nach Kursanleitung nachfüllen. → (4) Kabinenfenster von innen reinigen.</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F73" s="3" t="inlineStr">
-        <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
-      <c r="G73" s="3" t="inlineStr"/>
-      <c r="H73" s="3" t="inlineStr"/>
-      <c r="I73" s="3" t="inlineStr"/>
-      <c r="J73" s="3" t="inlineStr"/>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>IO Scanner / Ceramill Map DRS</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>(1) Siehe laminierte Anleitung. → (2) Scanner-Status prüfen (eingeschaltet, angemeldet)</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr"/>
+      <c r="H73" s="5" t="inlineStr"/>
+      <c r="I73" s="5" t="inlineStr"/>
+      <c r="J73" s="5" t="inlineStr"/>
     </row>
     <row r="74" ht="60" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>Gießen &amp; Strahlen</t>
+          <t>Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Drucktopf</t>
+          <t>KANBAN-Bestellung aufgeben</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>(1) ⚠ Den Drucktopf niemals ohne Einweisung bedienen – immer erst Druck vollständig ablassen!</t>
+          <t>(1) Karte an der KANBAN-Station im Sekretariat/ Koordination einlegen. → (2) Bearbeitung erfolgt automatisch.</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Werkstatt ZMK</t>
-        </is>
-      </c>
+          <t>Sekretariat / Koordination Skill Labs</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr"/>
       <c r="G74" s="4" t="inlineStr"/>
       <c r="H74" s="4" t="inlineStr"/>
       <c r="I74" s="4" t="inlineStr"/>
@@ -3152,12 +3152,12 @@
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Gießen &amp; Strahlen</t>
+          <t>Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Gerät defekt melden</t>
+          <t>Laptops für Aufsichten</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3167,17 +3167,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät außer Betrieb nehmen und kennzeichnen → (2) Reparaturauftrag ausfüllen (liegt im Technicum) → (3) Defekt mit kurzer Beschreibung melden</t>
+          <t>(1) Laptop im Sekretariat Skill Labs abholen. → (2) Einschalten und auf Funktionsfähigkeit prüfen. → (3) Nach dem Einsatz zurückgeben und zum laden einstecken.</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>Reparaturauftrag ausfüllen (liegt im Technicum) | Telefonliste ZMK – bei Dringlichkeit Mobilnr. | Techn. Koordinator in cc setzen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr"/>
@@ -3188,22 +3188,22 @@
     <row r="76" ht="60" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination</t>
+          <t>Papier &amp; Druck</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>IO Scanner / Ceramill Map DRS</t>
+          <t>Drucker</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>(1) Siehe laminierte Anleitung. → (2) Scanner-Status prüfen (eingeschaltet, angemeldet)</t>
+          <t>(1) Papierstau kann selbst behoben werden – Anleitung am Gerät. → (2) Tonerbestellung läuft automatisch. Kein Handlungsbedarf. (5) Fehlermeldung am Display notieren → (3) Hält der Defekt an → Druckerwartung melden → (4) Windows Startmenü öffnen → Ordner 90_Wartung. → (5) Drucker ZM11 (oder gewünschten Drucker) aus der Liste auswählen und installieren. → (6) Nach Installation: Drucker ggf. als Standard festlegen.</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Druckerwartung · Firma Morgenstern</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
@@ -3224,12 +3224,12 @@
     <row r="77" ht="60" customHeight="1">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination</t>
+          <t>Papier &amp; Druck</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>KANBAN-Bestellung aufgeben</t>
+          <t>Demoboxen</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3239,12 +3239,12 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>(1) Karte an der KANBAN-Station im Sekretariat/ Koordination einlegen. → (2) Bearbeitung erfolgt automatisch.</t>
+          <t>(1) Nur für den Prothetik-Kurs vorgesehen → (2) Entnahme/Rückgabe mit der Koordination abstimmen</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr"/>
@@ -3254,174 +3254,178 @@
       <c r="J77" s="3" t="inlineStr"/>
     </row>
     <row r="78" ht="60" customHeight="1">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>Laptops für Aufsichten</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>(1) Laptop im Sekretariat Skill Labs abholen. → (2) Einschalten und auf Funktionsfähigkeit prüfen. → (3) Nach dem Einsatz zurückgeben und zum laden einstecken.</t>
-        </is>
-      </c>
-      <c r="E78" s="4" t="inlineStr">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Besprechung Lehrende</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Küche &amp; Kaffee</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>(1) Mikrowelle, Kühlschrank und Kaffeevollautomat für Lehrende. Spül- und Reinigungsdienst für Tisch/Theke beachten – Organisation durch das Prothetik-Team.</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Die Steuerung für die Zentralabsauguing/ Trockenabsaugung befindet sich in diesem Raum</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79" ht="60" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Besprechung Lehrende</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>PC / Workstation – Funktionsstörung</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>IT-Service Tal</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr"/>
+    </row>
+    <row r="80" ht="60" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>CAD-Raum</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>3D-Scanner Pritimirror</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>(1) Software starten, Scanner einschalten – grüne Status-LED abwarten. → (2) Kalibrierung prüfen – Software meldet bei veralteter Kalibrierung. → (3) Scanfläche sauber halten – Staubpartikel verfälschen das Ergebnis. → (4) Modell fest positionieren – Bewegung während des Scans vermeiden.</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
-      <c r="G78" s="4" t="inlineStr"/>
-      <c r="H78" s="4" t="inlineStr"/>
-      <c r="I78" s="4" t="inlineStr"/>
-      <c r="J78" s="4" t="inlineStr"/>
-    </row>
-    <row r="79" ht="60" customHeight="1">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>Papier &amp; Druck</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>Drucker</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>mixed</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>(1) Papierstau kann selbst behoben werden – Anleitung am Gerät. → (2) Tonerbestellung läuft automatisch. Kein Handlungsbedarf. (5) Fehlermeldung am Display notieren → (3) Hält der Defekt an → Druckerwartung melden → (4) Windows Startmenü öffnen → Ordner 90_Wartung. → (5) Drucker ZM11 (oder gewünschten Drucker) aus der Liste auswählen und installieren. → (6) Nach Installation: Drucker ggf. als Standard festlegen.</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F79" s="5" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Druckerwartung · Firma Morgenstern</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="inlineStr"/>
-      <c r="H79" s="5" t="inlineStr"/>
-      <c r="I79" s="5" t="inlineStr"/>
-      <c r="J79" s="5" t="inlineStr"/>
-    </row>
-    <row r="80" ht="60" customHeight="1">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>Papier &amp; Druck</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>Demoboxen</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr">
-        <is>
-          <t>(1) Nur für den Prothetik-Kurs vorgesehen → (2) Entnahme/Rückgabe mit der Koordination abstimmen</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr"/>
-      <c r="G80" s="4" t="inlineStr"/>
-      <c r="H80" s="4" t="inlineStr"/>
-      <c r="I80" s="4" t="inlineStr"/>
-      <c r="J80" s="4" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
     </row>
     <row r="81" ht="60" customHeight="1">
-      <c r="A81" s="5" t="inlineStr">
-        <is>
-          <t>Besprechung Lehrende</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>Küche &amp; Kaffee</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>(1) Mikrowelle, Kühlschrank und Kaffeevollautomat für Lehrende. Spül- und Reinigungsdienst für Tisch/Theke beachten – Organisation durch das Prothetik-Team.</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>Die Steuerung für die Zentralabsauguing/ Trockenabsaugung befindet sich in diesem Raum</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="inlineStr"/>
-      <c r="H81" s="5" t="inlineStr"/>
-      <c r="I81" s="5" t="inlineStr"/>
-      <c r="J81" s="5" t="inlineStr"/>
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>CAD-Raum</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Creality Scan Ferret</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>(1) USB-Kabel fest einstecken – Treiber werden beim ersten Start installiert. → (2) Scanner parallel zur Oberfläche halten, gleichmäßig und ruhig bewegen. → (3) Tracking verloren? Scan pausieren, Gerät näher an Oberfläche führen, neu starten.</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr"/>
+      <c r="H81" s="3" t="inlineStr"/>
+      <c r="I81" s="3" t="inlineStr"/>
+      <c r="J81" s="3" t="inlineStr"/>
     </row>
     <row r="82" ht="60" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>Besprechung Lehrende</t>
+          <t>CAD-Raum</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>PC / Workstation – Funktionsstörung</t>
+          <t>Laborscanner Ceramill Map 300</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Software öffnen (Ceramill Map), Scanner einschalten – Verbindung abwarten. → (2) Modell auf den Scantisch legen – Referenzpunkte nicht verdecken. → (3) Kalibrierung: bei Aufforderung Kalibriermodell verwenden.</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -3430,40 +3434,40 @@
       <c r="J82" s="4" t="inlineStr"/>
     </row>
     <row r="83" ht="60" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>CAD-Raum</t>
         </is>
       </c>
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>3D-Scanner Pritimirror</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>(1) Software starten, Scanner einschalten – grüne Status-LED abwarten. → (2) Kalibrierung prüfen – Software meldet bei veralteter Kalibrierung. → (3) Scanfläche sauber halten – Staubpartikel verfälschen das Ergebnis. → (4) Modell fest positionieren – Bewegung während des Scans vermeiden.</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Haptic Pen (Geomagic Touch X)</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>(1) Gerät per USB anschließen, dann Software starten (nicht umgekehrt). → (2) Arm in Ruheposition (Dock) halten beim Starten der Software. → (3) Bewegungsbereich frei halten – Kabel nicht knicken oder verknoten. → (4) Kalibrierung: Anweisungen in der Software folgen wenn aufgefordert.</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
         <is>
           <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
-      <c r="F83" s="5" t="inlineStr">
+      <c r="F83" s="3" t="inlineStr">
         <is>
           <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
-      <c r="G83" s="5" t="inlineStr"/>
-      <c r="H83" s="5" t="inlineStr"/>
-      <c r="I83" s="5" t="inlineStr"/>
-      <c r="J83" s="5" t="inlineStr"/>
+      <c r="G83" s="3" t="inlineStr"/>
+      <c r="H83" s="3" t="inlineStr"/>
+      <c r="I83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="60" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
@@ -3473,27 +3477,23 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Creality Scan Ferret</t>
+          <t>Medienpanel / Raumsteuerung</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>(1) USB-Kabel fest einstecken – Treiber werden beim ersten Start installiert. → (2) Scanner parallel zur Oberfläche halten, gleichmäßig und ruhig bewegen. → (3) Tracking verloren? Scan pausieren, Gerät näher an Oberfläche führen, neu starten.</t>
-        </is>
-      </c>
+          <t>branch</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr"/>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Laborscanner Ceramill Map 300</t>
+          <t>Software startet nicht</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -3519,19 +3519,15 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>(1) Software öffnen (Ceramill Map), Scanner einschalten – Verbindung abwarten. → (2) Modell auf den Scantisch legen – Referenzpunkte nicht verdecken. → (3) Kalibrierung: bei Aufforderung Kalibriermodell verwenden.</t>
+          <t>(1) PC neu starten → (2) Software neu starten → (3) Lizenzserver erreichbar? → (4) Netzwerkverbindung prüfen (ist eine Eingabe der Proxydaten notwendig?)</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
-        </is>
-      </c>
-      <c r="F85" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr"/>
       <c r="G85" s="3" t="inlineStr"/>
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr"/>
@@ -3545,7 +3541,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Haptic Pen (Geomagic Touch X)</t>
+          <t>Lizenz nicht verfügbar</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -3555,19 +3551,15 @@
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>(1) Gerät per USB anschließen, dann Software starten (nicht umgekehrt). → (2) Arm in Ruheposition (Dock) halten beim Starten der Software. → (3) Bewegungsbereich frei halten – Kabel nicht knicken oder verknoten. → (4) Kalibrierung: Anweisungen in der Software folgen wenn aufgefordert.</t>
+          <t>(1) PC neu starten → (2) Prüfen ob die Netzwerk-/Serververbindung steht → (3) Software schließen und erneut öffnen</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="F86" s="4" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
+          <t>IT-Service Tal</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr"/>
       <c r="G86" s="4" t="inlineStr"/>
       <c r="H86" s="4" t="inlineStr"/>
       <c r="I86" s="4" t="inlineStr"/>
@@ -3581,23 +3573,27 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Medienpanel / Raumsteuerung</t>
+          <t>3D-Maus (3Dconnexion)</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D87" s="3" t="inlineStr"/>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>(1) USB-Stecker neu einstecken → (2) Anderen USB-Port testen → (3) Prüfen ob die 3Dconnexion-Software/Treiber läuft</t>
+        </is>
+      </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr"/>
@@ -3613,7 +3609,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Software startet nicht</t>
+          <t>Prusa Mini (3×)</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -3623,15 +3619,19 @@
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) Software neu starten → (3) Lizenzserver erreichbar? → (4) Netzwerkverbindung prüfen (ist eine Eingabe der Proxydaten notwendig?)</t>
+          <t>(1) Druckbett sauber und nivelliert? → (2) Filament vorhanden und korrekt eingezogen? → (3) Druckauftrag erneut senden</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F88" s="4" t="inlineStr"/>
+          <t>3D-Druck Mailbox</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
       <c r="G88" s="4" t="inlineStr"/>
       <c r="H88" s="4" t="inlineStr"/>
       <c r="I88" s="4" t="inlineStr"/>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Lizenz nicht verfügbar</t>
+          <t>IT / Netzwerkproblem</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) Prüfen ob die Netzwerk-/Serververbindung steht → (3) Software schließen und erneut öffnen</t>
+          <t>(1) PC neu starten → (2) Netzwerkkabel / Verbindung prüfen → (3) Über Windows-Menü auf 90_Wartung und dann Gruppenrichtlinie abrufen.</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
@@ -3663,7 +3663,11 @@
           <t>IT-Service Tal</t>
         </is>
       </c>
-      <c r="F89" s="3" t="inlineStr"/>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+        </is>
+      </c>
       <c r="G89" s="3" t="inlineStr"/>
       <c r="H89" s="3" t="inlineStr"/>
       <c r="I89" s="3" t="inlineStr"/>
@@ -3677,7 +3681,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>3D-Maus (3Dconnexion)</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -3687,17 +3691,17 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>(1) USB-Stecker neu einstecken → (2) Anderen USB-Port testen → (3) Prüfen ob die 3Dconnexion-Software/Treiber läuft</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: IT-Service Tal</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -3713,27 +3717,27 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Prusa Mini (3×)</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>(1) Druckbett sauber und nivelliert? → (2) Filament vorhanden und korrekt eingezogen? → (3) Druckauftrag erneut senden</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>3D-Druck Mailbox</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr"/>
@@ -3742,70 +3746,70 @@
       <c r="J91" s="3" t="inlineStr"/>
     </row>
     <row r="92" ht="60" customHeight="1">
-      <c r="A92" s="4" t="inlineStr">
-        <is>
-          <t>CAD-Raum</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>IT / Netzwerkproblem</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>(1) PC neu starten → (2) Netzwerkkabel / Verbindung prüfen → (3) Über Windows-Menü auf 90_Wartung und dann Gruppenrichtlinie abrufen.</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>IT-Service Tal</t>
-        </is>
-      </c>
-      <c r="F92" s="4" t="inlineStr">
-        <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
-        </is>
-      </c>
-      <c r="G92" s="4" t="inlineStr"/>
-      <c r="H92" s="4" t="inlineStr"/>
-      <c r="I92" s="4" t="inlineStr"/>
-      <c r="J92" s="4" t="inlineStr"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>CAM-Raum</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Ceramill Matik (Fräsmaschine)</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>safety</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Nur eingewiesene Personen dürfen die Ceramill Matik bedienen.</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
     </row>
     <row r="93" ht="60" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>CAD-Raum</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Buchung / Zugang</t>
+          <t>Ceramill Therm3 (Sinterofen)</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
+          <t>(1) ⚠ Nur eingewiesene Personen dürfen den Sinterofen bedienen.</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr"/>
@@ -3816,32 +3820,32 @@
     <row r="94" ht="60" customHeight="1">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>CAD-Raum</t>
+          <t>CAM-Raum</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>PC / Workstation – Funktionsstörung</t>
+          <t>xTool S1 Laser</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) ⚠ Schutzbrille Pflicht!  Nur eingewiesene Personen dürfen den Sinterofen bedienen..</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr"/>
@@ -3850,40 +3854,40 @@
       <c r="J94" s="4" t="inlineStr"/>
     </row>
     <row r="95" ht="60" customHeight="1">
-      <c r="A95" s="5" t="inlineStr">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>CAM-Raum</t>
         </is>
       </c>
-      <c r="B95" s="5" t="inlineStr">
-        <is>
-          <t>Ceramill Matik (Fräsmaschine)</t>
-        </is>
-      </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Nur eingewiesene Personen dürfen die Ceramill Matik bedienen.</t>
-        </is>
-      </c>
-      <c r="E95" s="5" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F95" s="5" t="inlineStr">
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Formlabs / Form Wash / Form Cure</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>(1) Resin vorhanden, Tank artefaktfrei? → (2) Wash-/Cure-Zeiten nach Anleitung einstellen → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
         <is>
           <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
         </is>
       </c>
-      <c r="G95" s="5" t="inlineStr"/>
-      <c r="H95" s="5" t="inlineStr"/>
-      <c r="I95" s="5" t="inlineStr"/>
-      <c r="J95" s="5" t="inlineStr"/>
+      <c r="G95" s="3" t="inlineStr"/>
+      <c r="H95" s="3" t="inlineStr"/>
+      <c r="I95" s="3" t="inlineStr"/>
+      <c r="J95" s="3" t="inlineStr"/>
     </row>
     <row r="96" ht="60" customHeight="1">
       <c r="A96" s="4" t="inlineStr">
@@ -3893,27 +3897,27 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Ceramill Therm3 (Sinterofen)</t>
+          <t>Bambu Lab / Prusa Mini</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>(1) ⚠ Nur eingewiesene Personen dürfen den Sinterofen bedienen.</t>
+          <t>(1) Druckbett sauber, Filament eingezogen? → (2) Druckauftrag auf SD Karte → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
         <is>
-          <t>Aufsichten / Ärzte im Raum</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -3929,27 +3933,27 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>xTool S1 Laser</t>
+          <t>KANBAN-Bestellung aufgeben</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>safety</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Schutzbrille Pflicht!  Nur eingewiesene Personen dürfen den Sinterofen bedienen..</t>
+          <t>(1) Karte ausfüllen und an KANBAN Station im Sekretariat/Koordination Skill Labs einlegen</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr"/>
@@ -3965,7 +3969,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Formlabs / Form Wash / Form Cure</t>
+          <t>Gefahrstoffentsorgung (IPA)</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -3975,17 +3979,17 @@
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>(1) Resin vorhanden, Tank artefaktfrei? → (2) Wash-/Cure-Zeiten nach Anleitung einstellen → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
+          <t>(1) Anmeldeformular Sonderabfälle ausfüllen (Anzahl / Art) → (2) Formular freitags an die Sonderabfall-Mailbox senden (Abholung dienstags) → (3) Etiketten bedrucken (IPA = halogenfreie Lösungsmittel) → (4) Kanister bekleben: UN-Nr. horizontal, Gefahrstoffkleber Spitze nach oben → (5) Kanister in Gefahrstoffcontainer OS8/LFB (Pfortenschlüssel im Sekretariat) → (6) Leere Kanister: ausdampfen, Symbol durchstreichen, ohne Deckel in gelben Sack</t>
         </is>
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Arbeitssicherheit</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Aufsichten / Ärzte im Raum</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -4001,7 +4005,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Bambu Lab / Prusa Mini</t>
+          <t>IT / Software</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4011,17 +4015,17 @@
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>(1) Druckbett sauber, Filament eingezogen? → (2) Druckauftrag auf SD Karte → (3) Für Druckaufträge: 3D-Druck-Mailbox kontaktieren</t>
+          <t>(1) PC neu starten → (2) An-/Abmeldung und Netzwerkverbindung prüfen → (3) Hält das Problem an → IT-Service Tal</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>IT-Service Tal</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr"/>
@@ -4037,27 +4041,27 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>KANBAN-Bestellung aufgeben</t>
+          <t>Unfall / Notfall</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>safety</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>(1) Karte ausfüllen und an KANBAN Station im Sekretariat/Koordination Skill Labs einlegen</t>
+          <t>(1) ⚠ Bei Verletzungen: Ärzte im Haus rufen, bei Bedarf Notarzt. SOP Unfallanzeige UKT beachten. Vorgesetzten informieren. Auge sofort an der Augendusche spülen, dabei aufhalten. Danach Arzt aufsuchen. Feuerlöscher: 1× Schaum. CO₂ bei Elektronik- und Flüssigkeitsbränden. Fluchtwege freihalten.</t>
         </is>
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
+          <t>Sofortmaßnahme</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Ärzte im Haus rufen, bei Bedarf Notarzt | SOP Unfallanzeige UKT beachten</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr"/>
@@ -4073,7 +4077,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Gefahrstoffentsorgung (IPA)</t>
+          <t>Buchung / Zugang</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -4083,17 +4087,17 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>(1) Anmeldeformular Sonderabfälle ausfüllen (Anzahl / Art) → (2) Formular freitags an die Sonderabfall-Mailbox senden (Abholung dienstags) → (3) Etiketten bedrucken (IPA = halogenfreie Lösungsmittel) → (4) Kanister bekleben: UN-Nr. horizontal, Gefahrstoffkleber Spitze nach oben → (5) Kanister in Gefahrstoffcontainer OS8/LFB (Pfortenschlüssel im Sekretariat) → (6) Leere Kanister: ausdampfen, Symbol durchstreichen, ohne Deckel in gelben Sack</t>
+          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>Technischer Koordinator Skill Labs</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G101" s="3" t="inlineStr"/>
@@ -4109,17 +4113,17 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>IT / Software</t>
+          <t>PC / Workstation – Funktionsstörung</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>(1) PC neu starten → (2) An-/Abmeldung und Netzwerkverbindung prüfen → (3) Hält das Problem an → IT-Service Tal</t>
+          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
@@ -4129,7 +4133,7 @@
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr"/>
@@ -4138,106 +4142,106 @@
       <c r="J102" s="4" t="inlineStr"/>
     </row>
     <row r="103" ht="60" customHeight="1">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>CAM-Raum</t>
-        </is>
-      </c>
-      <c r="B103" s="3" t="inlineStr">
-        <is>
-          <t>Unfall / Notfall</t>
-        </is>
-      </c>
-      <c r="C103" s="3" t="inlineStr">
-        <is>
-          <t>safety</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Bei Verletzungen: Ärzte im Haus rufen, bei Bedarf Notarzt. SOP Unfallanzeige UKT beachten. Vorgesetzten informieren. Auge sofort an der Augendusche spülen, dabei aufhalten. Danach Arzt aufsuchen. Feuerlöscher: 1× Schaum. CO₂ bei Elektronik- und Flüssigkeitsbränden. Fluchtwege freihalten.</t>
-        </is>
-      </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>Sofortmaßnahme</t>
-        </is>
-      </c>
-      <c r="F103" s="3" t="inlineStr">
-        <is>
-          <t>Ärzte im Haus rufen, bei Bedarf Notarzt | SOP Unfallanzeige UKT beachten</t>
-        </is>
-      </c>
-      <c r="G103" s="3" t="inlineStr"/>
-      <c r="H103" s="3" t="inlineStr"/>
-      <c r="I103" s="3" t="inlineStr"/>
-      <c r="J103" s="3" t="inlineStr"/>
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>LEAN · 3D-Druck · KANBAN</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>3D-Druck-Anfrage stellen</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D103" s="5" t="inlineStr">
+        <is>
+          <t>(1) STL-Datei vorbereiten (geschlossenes Volumen, korrekte Größe) → (2) Kurze Beschreibung + gewünschtes Material angeben → (3) An die 3D-Druck-Mailbox senden</t>
+        </is>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>3D-Druck Mailbox</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken</t>
+        </is>
+      </c>
+      <c r="G103" s="5" t="inlineStr"/>
+      <c r="H103" s="5" t="inlineStr"/>
+      <c r="I103" s="5" t="inlineStr"/>
+      <c r="J103" s="5" t="inlineStr"/>
     </row>
     <row r="104" ht="60" customHeight="1">
-      <c r="A104" s="4" t="inlineStr">
-        <is>
-          <t>CAM-Raum</t>
-        </is>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>Buchung / Zugang</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>(1) Verfügbarkeit im Routineraster / Google Kalender prüfen → (2) Freien Termin eintragen bzw. anfragen → (3) Zugang über die zuständige Stelle klären</t>
-        </is>
-      </c>
-      <c r="E104" s="4" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F104" s="4" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G104" s="4" t="inlineStr"/>
-      <c r="H104" s="4" t="inlineStr"/>
-      <c r="I104" s="4" t="inlineStr"/>
-      <c r="J104" s="4" t="inlineStr"/>
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Qualifizierung · Einweisung</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>CAD/CAM Sicherheitseinweisung</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
     </row>
     <row r="105" ht="60" customHeight="1">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>CAM-Raum</t>
+          <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>PC / Workstation – Funktionsstörung</t>
+          <t>Intraoralscanner (IOS) Einweisung</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>branch</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>(1) Alle Anwendungen schließen (falls möglich). → (2) PC über das Startmenü neu starten – nicht den Netzstecker ziehen. → (3) Falls kein Neustart möglich: Powerknopf 5 Sek. gedrückt halten. → (4) Nach Neustart prüfen, ob das Problem behoben ist. → (5) Kabel und Stecker prüfen (Monitor, Netzwerk, Strom). → (6) Fehlermeldung notieren und Screenshot erstellen.</t>
+          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>IT-Service Tal</t>
+          <t>Einweisung anfordern</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>Serviceportal oder Telefon – Telefonliste ZMK</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr"/>
@@ -4246,76 +4250,76 @@
       <c r="J105" s="3" t="inlineStr"/>
     </row>
     <row r="106" ht="60" customHeight="1">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>LEAN · 3D-Druck · KANBAN</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>3D-Druck-Anfrage stellen</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>(1) STL-Datei vorbereiten (geschlossenes Volumen, korrekte Größe) → (2) Kurze Beschreibung + gewünschtes Material angeben → (3) An die 3D-Druck-Mailbox senden</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>3D-Druck Mailbox</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>3DDruck@med.uni-tuebingen.de | STL-Datei + kurze Beschreibung mitschicken</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr"/>
-      <c r="I106" s="2" t="inlineStr"/>
-      <c r="J106" s="2" t="inlineStr"/>
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>Qualifizierung · Einweisung</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>Design-Prozess 4./5. Fachsemester</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>Einweisung anfordern</t>
+        </is>
+      </c>
+      <c r="F106" s="4" t="inlineStr">
+        <is>
+          <t>Zuständigen Kollegen ansprechen</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr"/>
+      <c r="H106" s="4" t="inlineStr"/>
+      <c r="I106" s="4" t="inlineStr"/>
+      <c r="J106" s="4" t="inlineStr"/>
     </row>
     <row r="107" ht="60" customHeight="1">
-      <c r="A107" s="5" t="inlineStr">
+      <c r="A107" s="3" t="inlineStr">
         <is>
           <t>Qualifizierung · Einweisung</t>
         </is>
       </c>
-      <c r="B107" s="5" t="inlineStr">
-        <is>
-          <t>CAD/CAM Sicherheitseinweisung</t>
-        </is>
-      </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
-        <is>
-          <t>(1) Termin für die Einweisung erfragen → (2) Ohne Einweisung keine Gerätenutzung</t>
-        </is>
-      </c>
-      <c r="E107" s="5" t="inlineStr">
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Schulungsvideos / Kompetenzmatrix</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>(1) Einführung in Adobe Premier Pro  (2) Einweisung in die Nutzung des Gimbals und de rAnsteckmikrofone</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
         <is>
           <t>Einweisung anfordern</t>
         </is>
       </c>
-      <c r="F107" s="5" t="inlineStr">
-        <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G107" s="5" t="inlineStr"/>
-      <c r="H107" s="5" t="inlineStr"/>
-      <c r="I107" s="5" t="inlineStr"/>
-      <c r="J107" s="5" t="inlineStr"/>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>siehe Kompetenzmatrix</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr"/>
+      <c r="H107" s="3" t="inlineStr"/>
+      <c r="I107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr"/>
     </row>
     <row r="108" ht="60" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
@@ -4325,7 +4329,7 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Intraoralscanner (IOS) Einweisung</t>
+          <t>Slicing / Nesting für Kurse</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -4335,7 +4339,7 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisungstermin erfragen → (2) Scanner erst nach Einweisung verwenden</t>
+          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
@@ -4345,7 +4349,7 @@
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr"/>
@@ -4361,7 +4365,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Design-Prozess 4./5. Fachsemester</t>
+          <t>Medientechnik</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -4371,7 +4375,7 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>(1) Kursunterlagen / Ablauf prüfen → (2) Bei Fragen zuständigen zahnärztlichen Kollegen ansprechen</t>
+          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
@@ -4381,7 +4385,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>Zuständigen Kollegen ansprechen</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr"/>
@@ -4397,7 +4401,7 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Schulungsvideos / Kompetenzmatrix</t>
+          <t>Haptic Device / 3D-Eingabestift</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -4407,7 +4411,7 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>(1) Einführung in Adobe Premier Pro  (2) Einweisung in die Nutzung des Gimbals und de rAnsteckmikrofone</t>
+          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
@@ -4417,7 +4421,7 @@
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>siehe Kompetenzmatrix</t>
+          <t>Arzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr"/>
@@ -4433,7 +4437,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Slicing / Nesting für Kurse</t>
+          <t>Einweisung KanbanSlides Excel</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -4443,7 +4447,7 @@
       </c>
       <c r="D111" s="3" t="inlineStr">
         <is>
-          <t>(1) Software/Vorlage nach Kursanleitung nutzen → (2) Bei Fragen Techn. Koordinator ansprechen</t>
+          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
@@ -4453,7 +4457,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>Zuständige Aufsicht oder Arzt im Raum ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr"/>
@@ -4469,7 +4473,7 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Medientechnik</t>
+          <t>KANBAN Materialverwaltung</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -4479,7 +4483,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisung in das Medienpanel / die Medientechnik erfragen</t>
+          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -4489,7 +4493,7 @@
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator ansprechen | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G112" s="4" t="inlineStr"/>
@@ -4498,70 +4502,70 @@
       <c r="J112" s="4" t="inlineStr"/>
     </row>
     <row r="113" ht="60" customHeight="1">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>Qualifizierung · Einweisung</t>
-        </is>
-      </c>
-      <c r="B113" s="3" t="inlineStr">
-        <is>
-          <t>Haptic Device / 3D-Eingabestift</t>
-        </is>
-      </c>
-      <c r="C113" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr">
-        <is>
-          <t>(1) USB-/Stromverbindung prüfen → (2) Software/Treiber gestartet? → (3) Bei Defekt → Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="E113" s="3" t="inlineStr">
-        <is>
-          <t>Einweisung anfordern</t>
-        </is>
-      </c>
-      <c r="F113" s="3" t="inlineStr">
-        <is>
-          <t>Arzt Skill Labs oder Techn. Koordinator – Einweisung anfordern | Falls nötig in CC / 2. Stelle: Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="G113" s="3" t="inlineStr"/>
-      <c r="H113" s="3" t="inlineStr"/>
-      <c r="I113" s="3" t="inlineStr"/>
-      <c r="J113" s="3" t="inlineStr"/>
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>Gebäude &amp; Infrastruktur</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Wasser</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="D113" s="5" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Hauptabsperrventil schließen, Bereich sichern. → (2) Betroffenen Bereich / Raum notieren. → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+        </is>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Werkstatt ZMK</t>
+        </is>
+      </c>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr"/>
+      <c r="H113" s="5" t="inlineStr"/>
+      <c r="I113" s="5" t="inlineStr"/>
+      <c r="J113" s="5" t="inlineStr"/>
     </row>
     <row r="114" ht="60" customHeight="1">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>Gebäude &amp; Infrastruktur</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Einweisung KanbanSlides Excel</t>
+          <t>Strom / Elektrik</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>(1) Einweisung beim Technischen Koordinator anfordern. → (2) Zugriff auf die KanbanSlides Excel-Datei klären.</t>
+          <t>(1) ⚠ Geräte ausschalten, Bereich verlassen wenn nötig. → (2) Sicherungskasten prüfen – ist eine Sicherung ausgelöst? → (3) Betroffenen Bereich / Gerät notieren. → (4) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E114" s="4" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
         </is>
       </c>
       <c r="G114" s="4" t="inlineStr"/>
@@ -4572,32 +4576,32 @@
     <row r="115" ht="60" customHeight="1">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>Qualifizierung · Einweisung</t>
+          <t>Gebäude &amp; Infrastruktur</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>KANBAN Materialverwaltung</t>
+          <t>Klimatisierung / Lüftung</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>self</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>(1) Bestände prüfen und KANBAN-Karten nachfüllen. → (2) Bestellungen über das KANBAN-System aufgeben. → (3) Bei Fragen zur Verwaltung Technischen Koordinator ansprechen.</t>
+          <t>(1) Betroffenen Raum und Art der Störung notieren (keine Kühlung, kein Luftstrom, Lärm, …). → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>Einweisung anfordern</t>
+          <t>Zuständige Stellen</t>
         </is>
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr"/>
@@ -4606,40 +4610,40 @@
       <c r="J115" s="3" t="inlineStr"/>
     </row>
     <row r="116" ht="60" customHeight="1">
-      <c r="A116" s="2" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>Gebäude &amp; Infrastruktur</t>
         </is>
       </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>Wasser</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Aufzug</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>(1) ⚠ Hauptabsperrventil schließen, Bereich sichern. → (2) Betroffenen Bereich / Raum notieren. → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>(1) ⚠ Ruhe bewahren – Person beruhigen, Notruf im Aufzug betätigen. → (2) Aufzug außer Betrieb kennzeichnen (Hinweis an der Tür). → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
         <is>
           <t>Werkstatt ZMK</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr">
-        <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
-        </is>
-      </c>
-      <c r="G116" s="2" t="inlineStr"/>
-      <c r="H116" s="2" t="inlineStr"/>
-      <c r="I116" s="2" t="inlineStr"/>
-      <c r="J116" s="2" t="inlineStr"/>
+      <c r="F116" s="4" t="inlineStr">
+        <is>
+          <t>Notrufknopf im Aufzug betätigen (direkte Verbindung zur Aufzugswartung) | TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen | Notruf 112 wenn keine andere Hilfe erreichbar</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr"/>
+      <c r="H116" s="4" t="inlineStr"/>
+      <c r="I116" s="4" t="inlineStr"/>
+      <c r="J116" s="4" t="inlineStr"/>
     </row>
     <row r="117" ht="60" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
@@ -4649,27 +4653,27 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Strom / Elektrik</t>
+          <t>Allgemeiner Defekt (Tür, Schloss, Mobiliar …)</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Geräte ausschalten, Bereich verlassen wenn nötig. → (2) Sicherungskasten prüfen – ist eine Sicherung ausgelöst? → (3) Betroffenen Bereich / Gerät notieren. → (4) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Defekt und genauen Ort (Raum, Tür, Möbel) kurz notieren. → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Zuständige Stellen</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr"/>
@@ -4685,7 +4689,7 @@
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Klimatisierung / Lüftung</t>
+          <t>Britta Wasserspender</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -4695,17 +4699,17 @@
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>(1) Betroffenen Raum und Art der Störung notieren (keine Kühlung, kein Luftstrom, Lärm, …). → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Gerät ausschalten. → (2) Art der Störung notieren (kein Wasser, Filterwechsel fällig, Leck, ...). → (3) Technischen Koordinator oder Sekretariat informieren.</t>
         </is>
       </c>
       <c r="E118" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Stellen</t>
+          <t>Werkstatt ZMK</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G118" s="4" t="inlineStr"/>
@@ -4721,7 +4725,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Aufzug</t>
+          <t>Brandschutztür</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4731,7 +4735,7 @@
       </c>
       <c r="D119" s="3" t="inlineStr">
         <is>
-          <t>(1) ⚠ Ruhe bewahren – Person beruhigen, Notruf im Aufzug betätigen. → (2) Aufzug außer Betrieb kennzeichnen (Hinweis an der Tür). → (3) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) ⚠ Brandschutztür nicht blockieren – Fluchtweg und Brandabschnitt müssen frei bleiben. → (2) Art des Problems notieren (schließt nicht vollständig, Geräusch, beschädigt, ...). → (3) TBA oder Werkstatt ZMK informieren.</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
@@ -4741,7 +4745,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>Notrufknopf im Aufzug betätigen (direkte Verbindung zur Aufzugswartung) | TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK / Mobilnr. bei Dringlichkeit | Technischer Koordinator Skill Labs – direkt ansprechen | Notruf 112 wenn keine andere Hilfe erreichbar</t>
+          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK | Technischer Koordinator Skill Labs – direkt ansprechen</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr"/>
@@ -4757,27 +4761,27 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Allgemeiner Defekt (Tür, Schloss, Mobiliar …)</t>
+          <t>Primion Schließsystem (Kartenzugang)</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>branch</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>(1) Defekt und genauen Ort (Raum, Tür, Möbel) kurz notieren. → (2) Eine der zuständigen Stellen informieren (siehe Ansprechpartner finden).</t>
+          <t>(1) Betroffenen Raum und Art des Defekts notieren. → (2) TBA oder IT-Service informieren.</t>
         </is>
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>Zuständige Stellen</t>
+          <t>Sekretariat / Koordination Skill Labs</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Reparaturauftrag ausfüllen (liegt im Technicum) | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
         </is>
       </c>
       <c r="G120" s="4" t="inlineStr"/>
@@ -4793,22 +4797,22 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>Britta Wasserspender</t>
+          <t>Flur E6 · Monitor – kein Bild</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>(1) Gerät ausschalten. → (2) Art der Störung notieren (kein Wasser, Filterwechsel fällig, Leck, ...). → (3) Technischen Koordinator oder Sekretariat informieren.</t>
+          <t>(1) Monitor eingeschaltet? → (2) Strom- und HDMI-Kabel geprüft?</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F121" s="3" t="inlineStr">
@@ -4829,141 +4833,33 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Brandschutztür</t>
+          <t>Flur E6 · Kalender wird nicht angezeigt</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>self</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>(1) ⚠ Brandschutztür nicht blockieren – Fluchtweg und Brandabschnitt müssen frei bleiben. → (2) Art des Problems notieren (schließt nicht vollständig, Geräusch, beschädigt, ...). → (3) TBA oder Werkstatt ZMK informieren.</t>
+          <t>(1) Bitte melden!</t>
         </is>
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>Werkstatt ZMK</t>
+          <t>Technischer Koordinator Skill Labs</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>TBA – Technisches Betriebsamt: 77171 | Werkstatt ZMK – Telefonliste ZMK | Technischer Koordinator Skill Labs – direkt ansprechen</t>
+          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
         </is>
       </c>
       <c r="G122" s="4" t="inlineStr"/>
       <c r="H122" s="4" t="inlineStr"/>
       <c r="I122" s="4" t="inlineStr"/>
       <c r="J122" s="4" t="inlineStr"/>
-    </row>
-    <row r="123" ht="60" customHeight="1">
-      <c r="A123" s="3" t="inlineStr">
-        <is>
-          <t>Gebäude &amp; Infrastruktur</t>
-        </is>
-      </c>
-      <c r="B123" s="3" t="inlineStr">
-        <is>
-          <t>Primion Schließsystem (Kartenzugang)</t>
-        </is>
-      </c>
-      <c r="C123" s="3" t="inlineStr">
-        <is>
-          <t>branch</t>
-        </is>
-      </c>
-      <c r="D123" s="3" t="inlineStr">
-        <is>
-          <t>(1) Betroffenen Raum und Art des Defekts notieren. → (2) TBA oder IT-Service informieren.</t>
-        </is>
-      </c>
-      <c r="E123" s="3" t="inlineStr">
-        <is>
-          <t>Sekretariat / Koordination Skill Labs</t>
-        </is>
-      </c>
-      <c r="F123" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Techn. Koordinator</t>
-        </is>
-      </c>
-      <c r="G123" s="3" t="inlineStr"/>
-      <c r="H123" s="3" t="inlineStr"/>
-      <c r="I123" s="3" t="inlineStr"/>
-      <c r="J123" s="3" t="inlineStr"/>
-    </row>
-    <row r="124" ht="60" customHeight="1">
-      <c r="A124" s="4" t="inlineStr">
-        <is>
-          <t>Gebäude &amp; Infrastruktur</t>
-        </is>
-      </c>
-      <c r="B124" s="4" t="inlineStr">
-        <is>
-          <t>Flur E6 · Monitor – kein Bild</t>
-        </is>
-      </c>
-      <c r="C124" s="4" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>(1) Monitor eingeschaltet? → (2) Strom- und HDMI-Kabel geprüft?</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr">
-        <is>
-          <t>Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="F124" s="4" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
-      <c r="G124" s="4" t="inlineStr"/>
-      <c r="H124" s="4" t="inlineStr"/>
-      <c r="I124" s="4" t="inlineStr"/>
-      <c r="J124" s="4" t="inlineStr"/>
-    </row>
-    <row r="125" ht="60" customHeight="1">
-      <c r="A125" s="3" t="inlineStr">
-        <is>
-          <t>Gebäude &amp; Infrastruktur</t>
-        </is>
-      </c>
-      <c r="B125" s="3" t="inlineStr">
-        <is>
-          <t>Flur E6 · Kalender wird nicht angezeigt</t>
-        </is>
-      </c>
-      <c r="C125" s="3" t="inlineStr">
-        <is>
-          <t>self</t>
-        </is>
-      </c>
-      <c r="D125" s="3" t="inlineStr">
-        <is>
-          <t>(1) Bitte melden!</t>
-        </is>
-      </c>
-      <c r="E125" s="3" t="inlineStr">
-        <is>
-          <t>Technischer Koordinator Skill Labs</t>
-        </is>
-      </c>
-      <c r="F125" s="3" t="inlineStr">
-        <is>
-          <t>Direkt ansprechen oder per Mail – cc: Sekretariat / Koordination</t>
-        </is>
-      </c>
-      <c r="G125" s="3" t="inlineStr"/>
-      <c r="H125" s="3" t="inlineStr"/>
-      <c r="I125" s="3" t="inlineStr"/>
-      <c r="J125" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>

</xml_diff>